<commit_message>
cập nhật: đồng bộ đặc tả tổng hợp quanly_khohang_v0.xlsx, đồng bộ json m1 m2 m3 và bổ sung bộ kiểm chứng chuyên sâu m2
</commit_message>
<xml_diff>
--- a/01_spec/quanly_khohang_v0.xlsx
+++ b/01_spec/quanly_khohang_v0.xlsx
@@ -42,7 +42,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -54,8 +54,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAEAEA"/>
-        <bgColor rgb="00EAEAEA"/>
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,16 +69,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
@@ -91,7 +91,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -497,7 +497,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Quy trình quản lý phiếu kho hàng điện máy gồm 6 hành vi: H1 tiếp nhận yêu cầu (chép mã phiếu vào bộ đệm), H2 tạo danh mục kiện hàng (cấp phát mảng sản phẩm trên heap), H3 tính tổng tiền tồn kho (số nguyên 32-bit, VND), H4 nhận ủy quyền thủ kho (chép token xác thực chữ ký), H5 ghi nhật ký kiểm kê kho (audit log), H6 đóng phiên kho hàng (worker nhập kho và worker xuất kho tự động dùng chung phiên). Bản v0 CÀI LỖI CÓ CHỦ ĐÍCH: 18 trường hợp rủi ro an toàn bộ nhớ và tràn số nguyên (15 lỗi ẩn) để kiểm chứng tính phát hiện của mô hình Kripke, Bounded Model Checking và AddressSanitizer.</t>
+          <t>Quy trình quản lý phiếu kho hàng điện máy gồm 6 hành vi: H1 tiếp nhận yêu cầu (chép mã phiếu vào bộ đệm Stack 32 byte - M1 Thọ), H2 tạo danh mục kiện hàng (cấp phát mảng struct Product trên Heap - M2 Trang), H3 tính tổng tiền và dung lượng mở rộng kho (số nguyên 32-bit, VND - M2/M3 Trang &amp; Đô), H4 nhận ủy quyền thủ kho và cộng dồn tồn kho (update_stock_quantity - M3 Đô), H5 ghi nhật ký kiểm kê và quy đổi đơn giá (scale_product_price - M3 Đô), H6 đóng phiên kho hàng (worker nhập kho và worker xuất kho tự động dùng chung phiên, thu hồi tài nguyên - M2 Trang). Bản v0 CÀI LỖI CÓ CHỦ ĐÍCH: 18 trường hợp rủi ro an toàn bộ nhớ và tràn số nguyên (15 lỗi ẩn) để kiểm chứng tính phát hiện của mô hình Kripke, Bounded Model Checking và AddressSanitizer.</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="61" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
@@ -574,24 +574,24 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu kho dài đúng 16 ký tự và dài 100 ký tự</t>
+          <t>Mã phiếu kho dài đúng 32 ký tự và dài 100 ký tự</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>parse_voucher_id sinh từ đặc tả (v0: Loi=buffer-overflow, buffer 16)</t>
+          <t>parse_voucher_id sinh từ đặc tả (v0: buffer 32 byte, Loi=buffer-overflow) - M1 Thọ</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Sinh mã C cho parse_voucher_id
 Chạy check_c_source() (Chương 2)
-Kiểm tra AG(!buffer_overflow), AG(!off_by_one) trên mô hình</t>
+Kiểm tra AG(!buffer_overflow), AG(!off_by_one) trên mô hình Kripke</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>v0: dangerous-function strcpy (CWE-120), 2 công thức VI PHẠM; v1: 0 phát hiện, công thức ĐÚNG</t>
+          <t>v0: dangerous-function strcpy (CWE-120/121), 2 công thức VI PHẠM; v1: 0 phát hiện, công thức ĐÚNG</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bản sửa của phần mềm có cắt cụt mã phiếu 16 ký tự không</t>
+          <t>Bản sửa của phần mềm có cắt cụt mã phiếu 32 ký tự không</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Mô hình con M1, luồng 'M1-v1a' (strncpy 15 + '\0')</t>
+          <t>Mô hình con M1, luồng 'M1-v1a' (strncpy 31 + '\0') - M1 Thọ</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Cấp phát mảng kiện hàng trên heap</t>
+          <t>Cấp phát mảng kiện hàng trên Heap</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>create_stock_items (alloc_release, không cài lỗi); mô hình con M2</t>
+          <t>create_stock_items (alloc_release); mô hình con M2 - M2 Trang</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Chạy check_c_source() trên mã sinh
 Kiểm tra M2-v0: AG(!null_deref), AG(!heap_overflow), AG(!uninit_read)
-Chạy KiemTraSoHoc alloc_bytes</t>
+Chạy KiemTraSoHoc heap_alloc_bytes</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Phần mềm quét mã: 0 phát hiện; mô hình M2-v0: 3 công thức VI PHẠM; alloc_bytes SAT (v0) / UNSAT (v1)</t>
+          <t>Phần mềm quét mã: 0 phát hiện; mô hình M2-v0: 3 công thức VI PHẠM; heap_alloc_bytes SAT (v0) / UNSAT (v1)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -691,18 +691,18 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Tổng giá trị tồn kho tràn int32</t>
+          <t>Tổng tiền tồn kho và cộng dồn tràn int32</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>KiemTraSoHoc stock_total_int32, line_amount_mul, accumulated_total; BMC vòng lặp trong file JSON</t>
+          <t>KiemTraSoHoc stock_addition_overflow, line_amount_mul, accumulated_total; BMC vòng lặp trong file JSON</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Chạy check_satisfiability() trên DieuKien
-Chạy BMC bmc_cong_don_kho_hang (k = 100)</t>
+Chạy BMC bmc_cong_don_ton_kho (k = 100)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -724,27 +724,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>REQ-07, CON-03</t>
+          <t>REQ-07, REQ-11, CON-03</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Giá trị tồn kho âm do chiết khấu</t>
+          <t>Số lượng nhập âm và số tiền âm do chiết khấu</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>KiemTraSoHoc negative_total</t>
+          <t>KiemTraSoHoc negative_quantity_check, negative_total - M3 Đô</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Chạy check_satisfiability() trên DieuKien</t>
+          <t>Chạy check_satisfiability() trên DieuKien của Z3</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>v0: SAT (vd discount &gt; subtotal); v1: UNSAT</t>
+          <t>v0: SAT (tìm được nghiệm added_quantity = -50 và discount &gt; subtotal); v1: UNSAT</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -766,12 +766,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Phân bổ chiết khấu với số kỳ = 0</t>
+          <t>Phân bổ chi phí kho với kỳ hạn = 0</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Hàm Python calc_discount_rate(total, rate) (kind = divide) — chỉ có ở v0</t>
+          <t>Hàm Python calc_batch_capacity(total_items, batch_size) (kind = divide) — chỉ có ở v0</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>v0: tìm được ít nhất 1 crash ZeroDivisionError (CWE-248/369); v1: hàm đã thay bằng kiểm tra 1 &lt;= rate &lt;= 24</t>
+          <t>v0: tìm được ít nhất 1 crash ZeroDivisionError (CWE-248/369); v1: hàm thay bằng kiểm tra 1 &lt;= batch_size &lt;= 24</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Token ủy quyền thủ kho dài hơn 20 ký tự</t>
+          <t>Mã token ủy quyền thủ kho dài hơn 20 ký tự</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>v0: dangerous-function (CWE-120); v1: 0 phát hiện</t>
+          <t>v0: dangerous-function strcpy (CWE-120); v1: 0 phát hiện</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -841,12 +841,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nhánh ẩn bỏ qua xác thực quyền thủ kho</t>
+          <t>Nhánh ẩn backdoor bỏ qua xác thực quyền thủ kho</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Hàm Python manager_auth_bypass(admin_id, pin_code), magic_values = (31337, 8080)</t>
+          <t>Hàm Python auth_debug_bypass(warehouse_id, debug_pin), magic_values = (31337, 8080)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -874,17 +874,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>REQ-11, NFR-03</t>
+          <t>REQ-12, NFR-03</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Rò rỉ bộ nhớ khi ghi nhật ký kiểm kê kho</t>
+          <t>Rò rỉ bộ nhớ khi mở rộng buffer ghi nhật ký kiểm kê</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>write_audit_log (v0: Loi=memory-leak)</t>
+          <t>write_inventory_log (v0: Loi=memory-leak)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -912,22 +912,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>REQ-12</t>
+          <t>REQ-13</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Chuỗi định dạng trong nhật ký kiểm kê</t>
+          <t>Chuỗi định dạng format string trong nhật ký kiểm kê</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mô hình con M5 — khuôn mẫu sinh mã của phần mềm không tạo được lỗi này</t>
+          <t>Mô hình con M5 (Ghi nhật ký kiểm kê kho)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Nạp mô hình con M5 vào tab Ch1
+          <t>Nạp M5_ghi_nhat_ky.json vào tab Ch1
 Chọn luồng M5-v0, kiểm tra AG(!format_string)
 Chọn luồng M5-v1, kiểm tra lại</t>
         </is>
@@ -951,12 +951,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>REQ-13, NFR-04</t>
+          <t>REQ-15, NFR-04</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Worker nhập kho và xuất kho cùng đóng phiên</t>
+          <t>Worker nhập kho và worker xuất kho tự động cùng đóng phiên</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Worker xuất kho tự động kích hoạt đúng lúc worker nhập kho đang giữ phiên
+          <t>Worker xuất kho kích hoạt đúng lúc worker nhập kho đang giữ phiên
 Chạy check_mutual_exclusion(model, 'nhap_locked', 'xuat_locked')</t>
         </is>
       </c>
@@ -989,28 +989,29 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>REQ-14, REQ-15</t>
+          <t>REQ-16, REQ-17</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Double free và use-after-free khi đóng phiên kho</t>
+          <t>Double-free và Use-after-free khi giải phóng phiên kho</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>close_inventory_session (double-free), release_item_buffer (use-after-free)</t>
+          <t>close_inventory_session (double-free), release_stock_items (use-after-free) - M2 Trang</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Gộp mã C của 2 hàm
-Chạy check_c_source()</t>
+Chạy check_c_source()
+Chạy kiểm toán AddressSanitizer</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>v0: double-free (CWE-415) và use-after-free (CWE-416); v1: 0 phát hiện</t>
+          <t>v0: double-free (CWE-415) và use-after-free (CWE-416); v1: 0 phát hiện, 0 crash ASan</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1027,22 +1028,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>REQ-16, NFR-05, CON-07</t>
+          <t>REQ-18, NFR-05, CON-07</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Mã PIN thủ kho còn trong bộ nhớ sau khi giải phóng</t>
+          <t>Mã PIN thủ kho còn trong bộ nhớ Heap sau khi giải phóng</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Mô hình con M6</t>
+          <t>Mô hình con M6 (Đóng phiên kho và thu hồi tài nguyên)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Nạp mô hình con M6 vào tab Ch1
+          <t>Nạp M6_dong_phien.json vào tab Ch1
 Chọn luồng M6-v0, kiểm tra AG(!secret_residue)
 Chọn luồng M6-v1, kiểm tra lại</t>
         </is>
@@ -1066,17 +1067,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>REQ-17, REQ-18</t>
+          <t>REQ-01 đến REQ-18</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Toàn luồng quản lý phiếu kho</t>
+          <t>Kiểm chứng toàn luồng quản lý kho hàng</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Mô hình kết hợp (sheet MoHinhTrangThai)</t>
+          <t>Mô hình kết hợp tổng thể (sheet MoHinhTrangThai 35 trạng thái)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1087,7 +1088,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Không deadlock; v0: AF(flow_end) và EF(input_rejected) VI PHẠM; v1: tất cả ĐÚNG</t>
+          <t>Không deadlock; v0: AF(flow_end) và EF(input_rejected) VI PHẠM; v1: tất cả 22 công thức ĐÚNG</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1112,7 +1113,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1146,7 +1147,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>H1: Hàm phân tích mã phiếu kho (parse_voucher_id) không được ghi vượt biên bộ đệm, kể cả khi mã dài ĐÚNG 16 ký tự (C1.2, C1.3)</t>
+          <t>H1: Hàm phân tích mã phiếu kho (parse_voucher_id) không được ghi vượt biên bộ đệm Stack 32 byte, kể cả khi mã dài ĐÚNG 32 ký tự (C1.2, C1.3)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1168,7 +1169,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>H1: Mã phiếu kho hợp lệ không được bị cắt cụt hoặc biến đổi khi lưu vào bộ đệm (C1.4)</t>
+          <t>H1: Mã phiếu kho hợp lệ không được bị cắt cụt hoặc biến đổi khi lưu vào bộ đệm Stack 32 byte (C1.4)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1190,7 +1191,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>H2: Kết quả cấp phát mảng kiện hàng (create_stock_items) phải được kiểm tra NULL trước khi sử dụng (C2.2)</t>
+          <t>H2: Kết quả cấp phát mảng kiện hàng động (create_stock_items) trên Heap phải được kiểm tra NULL trước khi sử dụng (C2.2)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1212,12 +1213,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>H2: Kích thước vùng nhớ cấp phát (số kiện x kích thước 1 kiện) không được tràn số hoặc âm (C2.3)</t>
+          <t>H2: Kích thước cấp phát mảng kiện hàng (n * sizeof(Product)) không được gây tràn số nguyên dẫn đến cấp phát thiếu bộ nhớ rồi ghi tràn Heap (C2.3)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1234,17 +1235,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>H2: Không được đọc trường dữ liệu của kiện hàng trước khi khởi tạo (C2.4)</t>
+          <t>H2: Mọi phần tử kiện hàng trong danh mục động phải được khởi tạo đầy đủ trước khi đọc, không đọc dữ liệu rác (C2.4)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>functional</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1257,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>H3: Tổng giá trị tồn kho không được tràn kiểu int32, kể cả khi cộng dồn nhiều dòng kiện hàng (C3.2, C3.3)</t>
+          <t>H3: Phép tính tổng giá trị tiền tồn kho (đơn giá x số lượng + phí đóng gói) không được gây tràn số nguyên có dấu 32-bit (C3.2, C3.3)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1278,7 +1279,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>H3: Số lượng tồn kho, đơn giá, chiết khấu không được âm; tổng giá trị phiếu kho không được âm (C3.4)</t>
+          <t>H3: Giá trị tiền tồn kho không được âm do chiết khấu lớn hơn tạm tính hoặc số lượng âm (C3.4)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1300,12 +1301,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>H3: Hàm tính tỷ lệ chiết khấu tồn kho không được gây lỗi không kiểm soát khi tỷ lệ/số kỳ = 0 (C3.5)</t>
+          <t>H3: Phép phân bổ định mức chi phí kho theo kỳ hạn không được chia cho 0 khi kỳ hạn bằng 0 (C3.5)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>functional</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1322,7 +1323,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>H4: Hàm phân tích token ủy quyền thủ kho (parse_auth_token) không được tràn bộ đệm (C4.2)</t>
+          <t>H4: Chuỗi mã token ủy quyền thủ kho từ nguồn ngoài không được vượt quá 20 ký tự (C4.2)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1344,12 +1345,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>H4: Mọi yêu cầu xuất nhập kho phải được xác thực chữ ký thủ kho; không được tồn tại nhánh ẩn bỏ qua kiểm tra (C4.3)</t>
+          <t>H4: Luồng xác thực quyền thủ kho không được chứa nhánh bí mật (magic value) bỏ qua kiểm tra an ninh (C4.3)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>security</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1366,17 +1367,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>H5: Bản ghi nhật ký kiểm kê kho (write_audit_log) phải được giải phóng trên mọi nhánh, kể cả nhánh lỗi (C5.2)</t>
+          <t>H4: Phép cộng dồn tồn kho mới vào tồn kho cũ (update_stock_quantity) không được gây tràn số nguyên có dấu 32-bit và phải từ chối số lượng nhập âm (C4.4)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1388,17 +1389,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>H5: Nội dung nhật ký kiểm kê có dữ liệu đầu vào không được dùng trực tiếp làm chuỗi định dạng của printf (C5.3)</t>
+          <t>H5: Hàm ghi nhật ký kiểm kê kho không được rò rỉ bộ nhớ tiến trình khi tái cấp phát bộ đệm nhật ký (C5.2)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1411,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>H6: Worker nhập kho và worker xuất kho tự động không được đồng thời giữ phiên quản lý kho (mutual exclusion) (C6.2)</t>
+          <t>H5: Nội dung ghi nhật ký kiểm kê không được sử dụng trực tiếp chuỗi do người dùng nhập làm format string cho printf/syslog (C5.3)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>security</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1432,17 +1433,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>H6: Phiên làm việc kho (close_inventory_session) chỉ được giải phóng đúng 1 lần (C6.3)</t>
+          <t>H5: Phép nhân quy đổi giá trị hàng hóa theo tỉ giá (scale_product_price) không được gây tràn số nguyên có dấu 32-bit (C5.4)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1454,12 +1455,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>H6: Không được truy cập phiên/bộ đệm kiện hàng (release_item_buffer) sau khi đã giải phóng (C6.4)</t>
+          <t>H6: Hai tiến trình worker nhập kho và worker xuất kho tự động dùng chung phiên kho không được đồng thời can thiệp gây tranh chấp tài nguyên (C6.2)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>concurrency</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1476,12 +1477,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>H6: Mã PIN xác thực thủ kho phải được xóa trắng bằng lệnh không bị trình biên dịch loại bỏ trước khi giải phóng (C6.5)</t>
+          <t>H6: Khi đóng phiên kho hàng, con trỏ phiên làm việc không được giải phóng hai lần (CWE-415 Double Free) (C6.3)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1498,12 +1499,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Toàn luồng: mọi đường xử lý quản lý kho cuối cùng phải kết thúc (thành công hoặc từ chối an toàn), không dừng ở trạng thái không an toàn</t>
+          <t>H6: Sau khi giải phóng bộ nhớ danh mục hàng hóa (release_stock_items), con trỏ phải được gán NULL ngay lập tức; cấm tuyệt đối đọc/ghi vào vùng nhớ đã giải phóng (CWE-416 Use-After-Free) (C6.4)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>liveness</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1520,17 +1521,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Toàn luồng: luồng cập nhật kho thành công phải đạt tới được (mô hình không tầm thường) và đầu vào xấu phải có nhánh từ chối</t>
+          <t>H6: Bộ nhớ chứa mã PIN thủ kho và dữ liệu nhạy cảm phải được xóa sạch bằng explicit_bzero trước khi gọi free(), không để sót lại trên Heap (C6.5)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>liveness</t>
+          <t>security</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1579,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống xử lý tối thiểu 300 giao dịch xuất nhập kho/giây trên phần cứng tham chiếu</t>
+          <t>Hệ thống xử lý tối thiểu 300 giao dịch xuất nhập kho/giây trên phần cứng máy chủ tham chiếu</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1595,7 +1596,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Phản hồi xác thực token ủy quyền thủ kho trong tối đa 2 giây (tránh timeout đồng bộ kho)</t>
+          <t>Phản hồi xác thực token ủy quyền thủ kho trong tối đa 2 giây (tránh timeout đồng bộ kho phân tán)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1629,12 +1630,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Phiên làm việc kho tự hết hạn sau 15 phút nếu không có thao tác tiếp theo (worker timeout)</t>
+          <t>Không xảy ra race condition giữa luồng nhập kho và luồng quét xuất kho tự động chu kỳ 15 phút</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1647,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Mã PIN xác thực và token thủ kho không được tồn tại trong bộ nhớ RAM quá thời gian hiệu lực phiên</t>
+          <t>Mã PIN thủ kho và token phiên làm việc không tồn tại trong dump bộ nhớ tiến trình sau khi đóng phiên kho</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1663,12 +1664,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nhật ký kiểm kê kho (audit log) được lưu trữ tối thiểu 24 tháng phục vụ thanh tra an toàn</t>
+          <t>Thời gian phản hồi thao tác mở rộng bộ nhớ danh mục hàng đạt trung bình O(1) thông qua chiến lược nhân đôi dung lượng</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1717,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu kho tối đa 16 ký tự ASCII (16 ký tự cần 17 byte kể cả '\0')</t>
+          <t>Mã phiếu kho tối đa 31 ký tự ASCII (31 ký tự cần 32 byte bộ đệm Stack kể cả '\0')</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1733,7 +1734,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mã token ủy quyền thủ kho tối đa 20 ký tự ASCII</t>
+          <t>Mã token ủy quyền thủ kho tối đa 20 ký tự ASCII (cần 21 byte kể cả '\0')</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1767,7 +1768,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Số tiền tính bằng VND; bản v0 dùng int 32-bit có dấu (tối đa 2.147.483.647); hạn mức 1 phiếu kho là 2.000.000.000 VND</t>
+          <t>Đơn giá và tổng tiền là số nguyên có dấu 32-bit (signed int, đơn vị VND)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1784,12 +1785,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Tỷ lệ phân bổ chiết khấu kho từ 1 đến 24 kỳ kiểm kê</t>
+          <t>Số kỳ hạn phân bổ định mức chi phí kho từ 1 đến 24 tháng</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1802,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Chỉ dùng thư viện chuẩn C; phiên làm việc kho được bảo vệ bằng cơ chế khóa phiên an toàn</t>
+          <t>Worker quét xuất kho tự động kích hoạt định kỳ sau 15 phút rảnh phiên</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1818,7 +1819,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Bộ đệm mã PIN xác thực 16 chữ số, chỉ tồn tại trong thời gian xử lý tác vụ kiểm kê</t>
+          <t>Bộ nhớ chứa mã PIN thủ kho và mảng kiện hàng động bắt buộc cấp phát trên Heap qua malloc/calloc</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1965,7 +1966,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu chép đủ, có '\0' (an toàn)</t>
+          <t>Mã phiếu chép đủ vào buffer 32 byte, có '\0' (an toàn)</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1979,7 @@
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>h1, buffer_overflow, off_by_one, violation</t>
+          <t>h1, stack_buffer_overflow, off_by_one, violation</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1993,7 +1994,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mã ĐÚNG 16 ký tự: strcpy ghi 17 byte, '\0' đè sang biến kề (lỗi ẩn)</t>
+          <t>Mã phiếu dài đúng 32 ký tự: ghi đè byte '\0' vào byte lân cận (lỗi ẩn Off-by-one)</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2007,7 @@
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>h1, buffer_overflow, violation</t>
+          <t>h1, stack_buffer_overflow, violation</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2021,7 +2022,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mã &gt; 16 ký tự: tràn bộ đệm stack</t>
+          <t>Mã phiếu dài &gt; 32 byte: ghi đè tràn stack frame (lỗi hiện Buffer Overflow)</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2050,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>items = malloc(n * sizeof(Item))</t>
+          <t>items = malloc(n * sizeof(Product))</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2078,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Cấp phát thành công và đã khởi tạo (an toàn)</t>
+          <t>Cấp phát thành công và đã khởi tạo struct (an toàn)</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2106,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>malloc trả NULL nhưng vẫn ghi vào (lỗi ẩn: chỉ khi cạn bộ nhớ)</t>
+          <t>malloc trả NULL khi hết RAM nhưng vẫn truy cập ghi vào (lỗi ẩn OOM)</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2134,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>n*48 tràn int32 hoặc n âm: cấp phát sai kích thước rồi ghi tràn heap (lỗi ẩn)</t>
+          <t>n*48 tràn int32 hoặc n âm: cấp phát sai kích thước rồi ghi tràn Heap (lỗi ẩn)</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2162,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Đọc status kiện hàng khi chưa khởi tạo (lỗi ẩn)</t>
+          <t>Đọc dữ liệu kiện hàng khi chưa khởi tạo memset/calloc (lỗi ẩn Uninit Read)</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2218,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Tổng giá trị tồn kho nằm trong miền hợp lệ (an toàn)</t>
+          <t>Tổng giá trị tồn kho nằm trong miền hợp lệ [0, 2 tỷ VND] (an toàn)</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2274,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>SL/chiết khấu âm hoặc chiết khấu &gt; tạm tính: tổng âm (lỗi ẩn)</t>
+          <t>SL/chiết khấu âm hoặc chiết khấu &gt; tạm tính: tổng tiền âm (lỗi ẩn)</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2302,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Phân bổ chiết khấu với kỳ hạn = 0: chia cho 0</t>
+          <t>Phân bổ chiết khấu với kỳ hạn = 0: chia cho 0 gây crash tiến trình</t>
         </is>
       </c>
     </row>
@@ -2314,12 +2315,12 @@
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>h4, token_received</t>
+          <t>h4, validating</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>h4_ok, h4_tu_choi_quyen, h4_tran_token, h4_nhanh_an</t>
+          <t>h4_ok, h4_tran_token, h4_nhanh_an, h4_tu_choi_quyen</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2329,7 +2330,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Nhận token ủy quyền từ thủ kho</t>
+          <t>Xác thực token ủy quyền thủ kho và cộng dồn số lượng tồn kho</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2343,7 @@
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>h4, token_verified</t>
+          <t>h4, token_ok, authorized</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2357,48 +2358,48 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Token hợp lệ, chữ ký đúng quyền thủ kho (an toàn)</t>
+          <t>Token hợp lệ, chữ ký đúng, cập nhật tồn kho an toàn</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>h4_tu_choi_quyen</t>
+          <t>h4_tran_token</t>
         </is>
       </c>
       <c r="B19" s="2" t="n"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>h4, token_rejected</t>
+          <t>h4, stack_buffer_overflow, violation</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>h6_phien_ranh</t>
+          <t>dung_khong_an_toan</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>C4.1</t>
+          <t>C4.2</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Token sai quyền bị từ chối (an toàn) — phiên do worker timeout đóng</t>
+          <t>Token ủy quyền dài &gt; 20 byte: ghi tràn bộ đệm token (lỗi hiện)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>h4_tran_token</t>
+          <t>h4_nhanh_an</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>h4, buffer_overflow, violation</t>
+          <t>h4, hidden_bypass, violation</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2408,40 +2409,40 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>C4.2</t>
+          <t>C4.3</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Token &gt; 20 ký tự: tràn bộ đệm</t>
+          <t>Token mang giá trị ma thuật (magic value 31337/8080) bỏ qua xác thực (cửa sau ẩn)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>h4_nhanh_an</t>
+          <t>h4_tu_choi_quyen</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>h4, hidden_bypass, violation</t>
+          <t>h4, token_invalid</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>dung_khong_an_toan</t>
+          <t>h6_phien_ranh</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>C4.3</t>
+          <t>C4.4</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Nhánh ẩn bỏ qua kiểm tra quyền thủ kho (31337, 8080) (lỗi ẩn)</t>
+          <t>Token sai: từ chối quyền nhưng vẫn đẩy phiên sang bước đóng (an toàn)</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2470,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>e = malloc(LogEntry); ghi nhật ký kiểm kê kho</t>
+          <t>Ghi nhật ký kiểm kê kho và quy đổi đơn giá sản phẩm</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2483,7 @@
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>h5, log_freed</t>
+          <t>h5, log_ok, audit_clean</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2497,7 +2498,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Ghi log kiểm kê xong và free(e) (an toàn)</t>
+          <t>Ghi log thành công, giải phóng bộ đệm log sạch sẽ</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2526,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Nhánh lỗi return sớm, quên free (lỗi ẩn: rò rỉ tích lũy)</t>
+          <t>realloc bộ đệm log thất bại gán đè NULL làm mất con trỏ cũ (CWE-401 rò rỉ bộ nhớ)</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2554,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>printf(msg) với msg chứa định dạng %x/%n (lỗi ẩn)</t>
+          <t>syslog(LOG_INFO, raw_comment): chuỗi nhập chứa %x/%n đọc ghi tùy ý bộ nhớ</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2582,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Phiên kho đang mở, chưa worker nào giữ</t>
+          <t>Phiên kho đang mở, chưa worker nào giữ khóa</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2610,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Worker nhập kho đang giữ phiên</t>
+          <t>Worker nhập kho đang giữ khóa phiên làm việc</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2638,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Worker xuất kho tự động (15 phút) đang giữ phiên</t>
+          <t>Worker xuất kho tự động (15 phút) đang giữ khóa phiên</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2666,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Cả 2 worker cùng giữ phiên (race condition, lỗi ẩn)</t>
+          <t>Cả 2 worker cùng giữ phiên (Race condition, vi phạm loại trừ lẫn nhau)</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2694,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Cả 2 worker cùng free(session) (lỗi ẩn)</t>
+          <t>Cả 2 worker cùng gọi free(session) trên cùng một con trỏ (CWE-415)</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2722,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Worker đến sau ghi vào phiên kho đã free (lỗi ẩn)</t>
+          <t>Worker đến sau đọc/ghi vào phiên kho đã bị worker trước free (CWE-416)</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2750,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Giải phóng bộ đệm mã PIN và phiên làm việc</t>
+          <t>Giải phóng bộ đệm mã PIN thủ kho và mảng sản phẩm</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2778,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Mã PIN thủ kho còn trong heap sau free (memset bị -O2 loại bỏ) (lỗi ẩn)</t>
+          <t>Mã PIN thủ kho còn nguyên trong Heap sau free (memset bị compiler tối ưu -O2 loại bỏ)</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2791,7 @@
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>flow_end, stock_done, mem_clean</t>
+          <t>flow_end, stock_done, mem_clean, safe</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2800,12 +2801,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>C6.1</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Kết thúc: đã xử lý phiếu kho, bộ nhớ sạch</t>
+          <t>Phiên kho kết thúc thành công, giải phóng toàn bộ bộ nhớ (trạng thái an toàn)</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2819,7 @@
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>flow_end, input_rejected, mem_clean</t>
+          <t>flow_end, input_rejected, mem_clean, safe</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2828,12 +2829,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>C1.4/C4.4</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Kết thúc: từ chối đầu vào xấu một cách an toàn</t>
+          <t>Từ chối đầu vào không hợp lệ, thu hồi bộ nhớ an toàn (v0 thiếu nhánh này)</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2847,7 @@
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>unsafe_halt</t>
+          <t>flow_end, unsafe_halt, violation</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2861,7 +2862,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái hút sau vi phạm (error location trong BMC)</t>
+          <t>Tiến trình sập (crash SIGSEGV/ABORT) do vi phạm an toàn bộ nhớ</t>
         </is>
       </c>
     </row>
@@ -2876,10 +2877,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2915,7 +2916,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Safety C1.2, C1.3, C4.2 — CWE-120/787</t>
+          <t>Safety C1.2, C1.3, C4.2 — CWE-120/787 (tràn stack bộ đệm mã phiếu 32 byte và token 20 byte)</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2928,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Safety C1.2 — CWE-193 (lỗi ẩn: mã đúng 16 ký tự)</t>
+          <t>Safety C1.2 — CWE-193 (lỗi ẩn: mã phiếu dài đúng 32 ký tự ghi đè null terminator)</t>
         </is>
       </c>
     </row>
@@ -2939,19 +2940,19 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Safety C2.2 — CWE-476/690</t>
+          <t>Safety C2.2 — CWE-476 (lỗi ẩn: malloc trả NULL khi cạn RAM nhưng vẫn ghi vào)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AG(!heap_overflow)</t>
+          <t>AG(!alloc_size_overflow)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Safety C2.3 — CWE-680/122</t>
+          <t>Safety C2.3 — CWE-190/787 (lỗi ẩn: n * 48 byte tràn int32 dẫn tới cấp phát thiếu ô nhớ trên Heap)</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2964,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Safety C2.4 — CWE-457/908</t>
+          <t>Safety C2.4 — CWE-457 (lỗi ẩn: đọc trường trạng thái kiện hàng khi chưa khởi tạo)</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2976,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Safety C3.2, C3.3 — CWE-190</t>
+          <t>Safety C3.2, C3.3, C4.4 — CWE-190 (lỗi ẩn: nhân đơn giá tràn int32 hoặc cộng dồn tồn kho vượt 2 tỷ)</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2988,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Safety C3.4 — CWE-191/839</t>
+          <t>Safety C3.4, C4.4 (lỗi ẩn: số lượng âm hoặc chiết khấu lớn hơn tạm tính làm tổng âm)</t>
         </is>
       </c>
     </row>
@@ -2999,7 +3000,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Safety C3.5 — CWE-369</t>
+          <t>Safety C3.5 — CWE-369 (lỗi crash: phân bổ chi phí kho với kỳ hạn bằng 0)</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3012,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Safety C4.3 — CWE-912/CWE-807</t>
+          <t>Safety C4.3 — CWE-912 (lỗi ẩn: token ma thuật 31337/8080 vượt mặt xác thực thủ kho)</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3024,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Safety C5.2 — CWE-401</t>
+          <t>Safety C5.2 — CWE-401 (lỗi ẩn: realloc thất bại gán đè NULL làm rò rỉ vùng nhớ tiến trình)</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3036,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Safety C5.3 — CWE-134</t>
+          <t>Safety C5.3 — CWE-134 (lỗi bảo mật: chuỗi format string trong ghi nhật ký kiểm kê)</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3048,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.2 — CWE-362/667</t>
+          <t>Safety C6.2 — CWE-667 (lỗi ẩn: worker nhập kho và worker xuất kho tự động cùng chiếm phiên)</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3060,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.3 — CWE-415</t>
+          <t>Safety C6.3 — CWE-415 (lỗi crash: giải phóng phiên kho 2 lần liên tiếp)</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3072,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.4 — CWE-416</t>
+          <t>Safety C6.4 — CWE-416 (lỗi ẩn: đọc/ghi dữ liệu sau khi đã gọi free phiên kho)</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3084,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.5 — CWE-226/CWE-14</t>
+          <t>Safety C6.5 — CWE-226/14 (lỗi ẩn: mã PIN thủ kho còn sót lại trên Heap sau khi giải phóng)</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3096,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Liveness REQ-17: mọi lượt xử lý đều kết thúc hợp lệ</t>
+          <t>Liveness: mọi nhánh xử lý đều kết thúc (v0 kẹt tại trạng thái vi phạm lặp vô tận)</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3108,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Khả đạt REQ-18: tồn tại đường đi cập nhật kho thành công</t>
+          <t>Khả đạt REQ-18: tồn tại đường đi hoàn thành phiên kho an toàn thành công</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3120,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Khả đạt REQ-18: tồn tại nhánh từ chối đầu vào xấu (v0 KHÔNG có -&gt; VI PHẠM)</t>
+          <t>Khả đạt: tồn tại nhánh từ chối đầu vào độc hại/sai cú pháp (v0 KHÔNG có -&gt; VI PHẠM)</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3132,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tồn tại ít nhất 1 đường đi luôn an toàn</t>
+          <t>Tồn tại ít nhất một đường đi luôn an toàn từ đầu đến cuối</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3144,19 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Khả đạt của cụm khóa phiên (mô hình khóa không tầm thường)</t>
+          <t>Khả đạt của cụm khóa phiên nhập kho (mô hình khóa phiên hoạt động được)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>EF(xuat_locked)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Khả đạt của cụm khóa phiên xuất kho tự động (mô hình khóa phiên hoạt động được)</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -3232,6 +3245,18 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>mem_clean</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>secret_residue</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>mem_clean</t>
         </is>
@@ -3248,13 +3273,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
@@ -3331,7 +3356,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -3342,7 +3367,7 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>H1 — C1.2/C1.3 (CON-01)</t>
+          <t>H1 — C1.2/C1.3 (CON-01 bộ đệm Stack 32 byte - M1 Thọ)</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3404,7 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>H4 — C4.2 (CON-02)</t>
+          <t>H4 — C4.2 (CON-02 token 20 byte)</t>
         </is>
       </c>
     </row>
@@ -3408,14 +3433,14 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>H2 — phần mềm báo SẠCH nhưng mô hình chỉ ra C2.2/C2.3/C2.4 (tầng 2)</t>
+          <t>H2 — C2.2/C2.3/C2.4 cấp phát động struct Product trên Heap (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>write_audit_log</t>
+          <t>expand_stock_items</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -3430,7 +3455,7 @@
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -3441,14 +3466,14 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>H5 — C5.2</t>
+          <t>H3 — realloc mảng động khi OOM làm mất con trỏ gốc (CWE-401 - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>close_inventory_session</t>
+          <t>release_stock_items</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3463,25 +3488,25 @@
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>double-free</t>
+          <t>use-after-free</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>H6 — C6.3</t>
+          <t>H6 — free() không gán NULL dẫn tới Use-After-Free (CWE-416 - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>release_item_buffer</t>
+          <t>write_inventory_log</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -3496,25 +3521,25 @@
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>use-after-free</t>
+          <t>memory-leak</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>H6 — C6.4 (CON-07)</t>
+          <t>H5 — C5.2 rò rỉ bộ nhớ khi mở rộng buffer log</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>add_packing_fee</t>
+          <t>close_inventory_session</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3524,43 +3549,45 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>arithmetic</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>subtotal, packing_fee</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+          <t>alloc_release</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>double-free</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>H3 — trích AST cho Chương 3</t>
+          <t>H6 — C6.3 giải phóng phiên làm việc hai lần (CWE-415)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>calc_discount_rate</t>
+          <t>update_stock_quantity</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>divide</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>total, rate</t>
+          <t>current_stock, added_quantity</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
@@ -3569,42 +3596,104 @@
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>H3 — C3.5 (black-box fuzz)</t>
+          <t>H4 — C4.4 cộng dồn tồn kho tràn signed int 32-bit (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>manager_auth_bypass</t>
+          <t>scale_product_price</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>magic_value</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>admin_id, pin_code</t>
+          <t>base_price, rate</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>H5 — C5.4 nhân tỉ giá quy đổi tràn int32 (M3 Đô)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>calc_batch_capacity</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>divide</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>total_items, batch_size</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>H3 — C3.5 chia cho 0 khi batch_size = 0 (black-box fuzz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>auth_debug_bypass</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>magic_value</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>warehouse_id, debug_pin</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n">
         <v>31337</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>8080</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>H4 — C4.3 nhánh ẩn (concolic)</t>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>H4 — C4.3 nhánh ẩn backdoor vượt mặt xác thực (concolic)</t>
         </is>
       </c>
     </row>
@@ -3619,14 +3708,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="61" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3659,135 +3748,162 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>stock_total_int32</t>
+          <t>stock_addition_overflow</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>subtotal, packing_fee</t>
+          <t>current_stock, added_quantity</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>subtotal &gt;= 0 and subtotal &lt;= 2147483647 and packing_fee &gt;= 0 and packing_fee &lt;= 500000 and subtotal + packing_fee &gt; 2147483647</t>
+          <t>current_stock &gt;= 0 and current_stock &lt;= 2147483647 and added_quantity &gt;= 1 and added_quantity &lt;= 2147483647 and current_stock + added_quantity &gt; 2147483647</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>subtotal + packing_fee</t>
+          <t>current_stock + added_quantity</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>C3.2 — cộng phí đóng gói vào tạm tính gần trần int32</t>
+          <t>C4.4 — phép cộng dồn tồn kho mới vào tồn kho cũ vượt trần INT_MAX (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>line_amount_mul</t>
+          <t>heap_alloc_bytes</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>price, qty</t>
+          <t>new_capacity, item_size</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>price &gt;= 0 and price &lt;= 50000000 and qty &gt;= 1 and qty &lt;= 1000 and price * qty &gt; 2147483647</t>
+          <t>new_capacity &gt;= 1 and item_size == 48 and new_capacity * item_size &gt; 2147483647</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>price * qty</t>
+          <t>new_capacity * item_size</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C3.2 — phép nhân tràn TRƯỚC khi kịp kiểm tra hạn mức dòng</t>
+          <t>C2.3 — kích thước tái cấp phát Heap vượt 2GB khi new_capacity lớn (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>accumulated_total</t>
+          <t>line_amount_mul</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>total_before, line_total</t>
+          <t>price, qty</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>total_before &gt;= 0 and total_before &lt;= 2147483647 and line_total &gt;= 0 and line_total &lt;= 50000000 and total_before + line_total &gt; 2147483647</t>
+          <t>price &gt;= 0 and price &lt;= 50000000 and qty &gt;= 1 and qty &lt;= 1000 and price * qty &gt; 2147483647</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>total_before + line_total</t>
+          <t>price * qty</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>C3.3 — bước cộng dồn: mỗi dòng hợp lệ nhưng tổng vượt trần</t>
+          <t>C3.2 — phép nhân đơn giá x số lượng tràn TRƯỚC khi kịp kiểm tra hạn mức dòng</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>alloc_bytes</t>
+          <t>accumulated_total</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>n_items, item_size</t>
+          <t>total_before, line_total</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>n_items &gt;= 1 and item_size == 48 and n_items * item_size &gt; 2147483647</t>
+          <t>total_before &gt;= 0 and total_before &lt;= 2147483647 and line_total &gt;= 0 and line_total &lt;= 50000000 and total_before + line_total &gt; 2147483647</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>n_items * item_size</t>
+          <t>total_before + line_total</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>C2.3 — kích thước cấp phát tràn khi n không bị giới hạn</t>
+          <t>C3.3 — bước cộng dồn nhiều kiện hàng: mỗi kiện hợp lệ nhưng tổng vượt trần int32</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>negative_quantity_check</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>added_quantity</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>added_quantity &lt; 0</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>added_quantity</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>C4.4 — số lượng nhập hàng là số âm làm sai lệch số liệu kho (M3 Đô)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>negative_total</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>subtotal, discount</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>subtotal &gt;= 0 and subtotal &lt;= 2000000000 and discount + 2000000000 &gt;= 0 and discount &lt;= 2000000000 and subtotal - discount &lt; 0</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>subtotal - discount</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>C3.4 — chiết khấu âm hoặc lớn hơn tạm tính</t>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>C3.4 — chiết khấu giảm giá âm hoặc lớn hơn tạm tính làm tổng tiền âm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cập nhật đặc tả: chuẩn hóa m1 khớp với m2 m3 và đồng bộ toàn diện h1 nạp chuỗi và h2 đọc token trên excel json
</commit_message>
<xml_diff>
--- a/01_spec/quanly_khohang_v0.xlsx
+++ b/01_spec/quanly_khohang_v0.xlsx
@@ -497,7 +497,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Quy trình quản lý phiếu kho hàng điện máy gồm 6 hành vi: H1 tiếp nhận yêu cầu (chép mã phiếu vào bộ đệm Stack 32 byte - M1 Thọ), H2 tạo danh mục kiện hàng (cấp phát mảng struct Product trên Heap - M2 Trang), H3 tính tổng tiền và dung lượng mở rộng kho (số nguyên 32-bit, VND - M2/M3 Trang &amp; Đô), H4 nhận ủy quyền thủ kho và cộng dồn tồn kho (update_stock_quantity - M3 Đô), H5 ghi nhật ký kiểm kê và quy đổi đơn giá (scale_product_price - M3 Đô), H6 đóng phiên kho hàng (worker nhập kho và worker xuất kho tự động dùng chung phiên, thu hồi tài nguyên - M2 Trang). Bản v0 CÀI LỖI CÓ CHỦ ĐÍCH: 18 trường hợp rủi ro an toàn bộ nhớ và tràn số nguyên (15 lỗi ẩn) để kiểm chứng tính phát hiện của mô hình Kripke, Bounded Model Checking và AddressSanitizer.</t>
+          <t>Quy trình quản lý phiếu kho hàng điện máy gồm 6 hành vi của 3 thành viên: H1 nạp chuỗi mã phiếu kho vào bộ đệm Stack 32 byte (ingest_raw_line - M1 Nguyễn Quang Thọ), H2 đọc trường dữ liệu token theo chỉ số mảng (get_token_field - M1 Nguyễn Quang Thọ), H3 mở rộng động danh mục hàng hóa trên Heap khi danh sách đầy (expand_stock_items - M2 Nguyễn Kiều Trang), H4 cộng dồn số lượng tồn kho mới vào tồn kho cũ (update_stock_quantity - M3 Hà Văn Đô), H5 quy đổi đơn giá sản phẩm theo tỉ giá (scale_product_price - M3 Hà Văn Đô), H6 thu hồi tài nguyên và đóng phiên kho (release_stock_items - M2 Nguyễn Kiều Trang). Bản v0 CÀI LỖI CÓ CHỦ ĐÍCH: 18 trường hợp rủi ro an toàn bộ nhớ (CWE-120/121 Stack Overflow, CWE-193 Off-by-one, CWE-125 Out-of-bounds Read, CWE-401 Memory Leak, CWE-416 Use-After-Free, CWE-415 Double Free) và tràn số nguyên (CWE-190) để kiểm chứng tính phát hiện của mô hình Kripke, BMC và AddressSanitizer.</t>
         </is>
       </c>
     </row>
@@ -512,12 +512,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="61" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
@@ -574,24 +574,23 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu kho dài đúng 32 ký tự và dài 100 ký tự</t>
+          <t>H1: Nạp chuỗi đúng 32 byte gây lỗi Off-by-one và 33 byte tràn stack</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>parse_voucher_id sinh từ đặc tả (v0: buffer 32 byte, Loi=buffer-overflow) - M1 Thọ</t>
+          <t>ingest_raw_line sinh từ đặc tả (v0: buffer 32 byte, Loi=buffer-overflow) - M1 Thọ</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sinh mã C cho parse_voucher_id
-Chạy check_c_source() (Chương 2)
-Kiểm tra AG(!buffer_overflow), AG(!off_by_one) trên mô hình Kripke</t>
+          <t>Gọi ingest_raw_line_v0 với chuỗi 32 và 33 ký tự
+Chạy kiểm tra AG(!stack_buffer_overflow), AG(!off_by_one)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>v0: dangerous-function strcpy (CWE-120/121), 2 công thức VI PHẠM; v1: 0 phát hiện, công thức ĐÚNG</t>
+          <t>v0: ghi đè byte '\0' và tràn stack frame (CWE-120/121, CWE-193); v1: rào chắn từ chối trả về -2</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -613,24 +612,23 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bản sửa của phần mềm có cắt cụt mã phiếu 32 ký tự không</t>
+          <t>H1: Nạp chuỗi hợp lệ 31 byte vào bộ đệm stack 32 byte</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Mô hình con M1, luồng 'M1-v1a' (strncpy 31 + '\0') - M1 Thọ</t>
+          <t>char buffer[32], cap = 32, chuỗi đầu vào dài đúng 31 ký tự - M1 Thọ</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nạp mo_hinh_con/m1_doc_chuoi_buffer.json vào tab Ch1
-Chọn luồng M1-v1a, kiểm tra AG(!truncated)
-So sánh với luồng M1-v1b</t>
+          <t>Gọi v0 và v1 với chuỗi 31 byte
+Kiểm tra giá trị trả về và nội dung bộ đệm</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>M1-v1a: AG(!truncated) VI PHẠM (mã bị cắt, phần mềm không báo); M1-v1b: ĐÚNG</t>
+          <t>Cả 2 phiên bản trả về 31, sao chép thành công có '\0'</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -647,29 +645,28 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>REQ-03, REQ-04, REQ-05</t>
+          <t>REQ-03, CON-02</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Cấp phát mảng kiện hàng trên Heap</t>
+          <t>H2: Đọc token tại chỉ số chạm biên trên field_idx == token_count</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>create_stock_items (alloc_release); mô hình con M2 - M2 Trang</t>
+          <t>token_offsets có 4 phần tử (chỉ số 0..3), field_idx = 4 - M1 Thọ</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chạy check_c_source() trên mã sinh
-Kiểm tra M2-v0: AG(!null_deref), AG(!heap_overflow), AG(!uninit_read)
-Chạy KiemTraSoHoc heap_alloc_bytes</t>
+          <t>Gọi get_token_field_v0 với field_idx = 4 dưới giám sát ASan
+Gọi get_token_field_v1 với cùng tham số</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Phần mềm quét mã: 0 phát hiện; mô hình M2-v0: 3 công thức VI PHẠM; heap_alloc_bytes SAT (v0) / UNSAT (v1)</t>
+          <t>v0: Đọc ngoài biên mảng token (CWE-125); v1: Rào chắn chặn trả về -2</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -686,28 +683,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>REQ-06, CON-03, CON-04</t>
+          <t>REQ-04, CON-02</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Tổng tiền tồn kho và cộng dồn tràn int32</t>
+          <t>H2: Đọc token với chỉ số âm field_idx &lt; 0</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>KiemTraSoHoc stock_addition_overflow, line_amount_mul, accumulated_total; BMC vòng lặp trong file JSON</t>
+          <t>token_count = 4, field_idx = -1 - M1 Thọ</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chạy check_satisfiability() trên DieuKien
-Chạy BMC bmc_cong_don_ton_kho (k = 100)</t>
+          <t>Gọi get_token_field_v0 với field_idx = -1
+Gọi đối chứng get_token_field_v1</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>v0: SAT kèm phản ví dụ, BMC vi phạm tại bước 48 (total = 2.160.000.000); v1: UNSAT, BMC không vi phạm</t>
+          <t>v0: Đọc lùi vùng nhớ trước mảng (CWE-125); v1: Từ chối an toàn trả về -2</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -724,27 +721,28 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>REQ-07, REQ-11, CON-03</t>
+          <t>REQ-05, CON-03</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Số lượng nhập âm và số tiền âm do chiết khấu</t>
+          <t>H3: Mô phỏng sự cố OOM khi realloc mảng danh mục hàng</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>KiemTraSoHoc negative_quantity_check, negative_total - M3 Đô</t>
+          <t>realloc trả về NULL khi hệ thống cạn kiệt RAM - M2 Trang</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Chạy check_satisfiability() trên DieuKien của Z3</t>
+          <t>Gọi expand_stock_items trên bản v0 và v1 khi mảng đầy cần nhân đôi
+Quan sát con trỏ list</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>v0: SAT (tìm được nghiệm added_quantity = -50 và discount &gt; subtotal); v1: UNSAT</t>
+          <t>v0: list bị gán NULL làm mất địa chỉ mảng cũ (CWE-401 Leak); v1: giữ nguyên con trỏ cũ qua biến tạm tmp</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -761,32 +759,33 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>REQ-08, CON-05</t>
+          <t>REQ-06, CON-03</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Phân bổ chi phí kho với kỳ hạn = 0</t>
+          <t>H3: Tràn số nguyên khi tính toán kích thước mở rộng mảng động</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Hàm Python calc_batch_capacity(total_items, batch_size) (kind = divide) — chỉ có ở v0</t>
+          <t>new_capacity lớn gây tràn phép nhân new_capacity * sizeof(Product) - M2 Trang</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Chạy blackbox_fuzz() 300 lần</t>
+          <t>Chạy kiểm tra SMT Z3 trên điều kiện heap_alloc_bytes
+Thực thi hàm mở rộng</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>v0: tìm được ít nhất 1 crash ZeroDivisionError (CWE-248/369); v1: hàm thay bằng kiểm tra 1 &lt;= batch_size &lt;= 24</t>
+          <t>v0: SAT (tìm được nghiệm tràn int32 cấp phát thiếu ô nhớ); v1: UNSAT</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -798,28 +797,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>REQ-09, CON-02</t>
+          <t>REQ-07, CON-04</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Mã token ủy quyền thủ kho dài hơn 20 ký tự</t>
+          <t>H4: Cộng dồn số lượng tồn kho mới vượt trần INT_MAX</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>parse_auth_token (v0: buffer 20, Loi=buffer-overflow)</t>
+          <t>current_stock = 2.147.483.640, added_quantity = 20 - M3 Đô</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sinh mã C
-Chạy check_c_source()</t>
+          <t>Gọi update_stock_quantity trên bản v0 và v1</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>v0: dangerous-function strcpy (CWE-120); v1: 0 phát hiện</t>
+          <t>v0: 2147483640 + 20 = -2147483636 (tràn số âm CWE-190); v1: từ chối trước khi cộng</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -836,28 +834,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>REQ-10</t>
+          <t>REQ-08, CON-04</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nhánh ẩn backdoor bỏ qua xác thực quyền thủ kho</t>
+          <t>H4: Số lượng nhập hàng là số âm (added_quantity &lt; 0)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Hàm Python auth_debug_bypass(warehouse_id, debug_pin), magic_values = (31337, 8080)</t>
+          <t>added_quantity = -50 - M3 Đô</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Chạy black-box fuzz trước (kỳ vọng không tìm ra)
-Chạy concolic_fuzz()</t>
+          <t>Gọi update_stock_quantity với số lượng âm</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Black-box: 0 lần chạm nhánh; concolic: tìm đúng (31337, 8080) sau vài lần thử (CWE-912)</t>
+          <t>v0: trừ lùi tồn kho sai nghiệp vụ; v1: phát hiện số âm từ chối an toàn</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -874,33 +871,32 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>REQ-12, NFR-03</t>
+          <t>REQ-09, CON-04</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Rò rỉ bộ nhớ khi mở rộng buffer ghi nhật ký kiểm kê</t>
+          <t>H5: Quy đổi đơn giá sản phẩm theo tỉ giá gây tràn phép nhân</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>write_inventory_log (v0: Loi=memory-leak)</t>
+          <t>base_price = 50.000.000, rate = 100 - M3 Đô</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Sinh mã C
-Chạy check_c_source()</t>
+          <t>Gọi scale_product_price trên bản v0 và v1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>v0: memory-leak (CWE-401); v1: 0 phát hiện</t>
+          <t>v0: 50.000.000 * 100 vượt INT_MAX gây tràn số (CWE-190); v1: rào chắn từ chối an toàn</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -912,34 +908,32 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>REQ-13</t>
+          <t>REQ-10, CON-05</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Chuỗi định dạng format string trong nhật ký kiểm kê</t>
+          <t>H6: Tranh chấp khóa phiên giữa worker nhập kho và xuất kho</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mô hình con M5 (Ghi nhật ký kiểm kê kho)</t>
+          <t>Cả 2 worker cùng giữ phiên làm việc tại h6_tranh_chap - M2 Trang</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Nạp M5_ghi_nhat_ky.json vào tab Ch1
-Chọn luồng M5-v0, kiểm tra AG(!format_string)
-Chọn luồng M5-v1, kiểm tra lại</t>
+          <t>Chạy check_mutual_exclusion(model, 'nhap_locked', 'xuat_locked')</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>M5-v0: AG(!format_string) VI PHẠM (CWE-134); M5-v1: ĐÚNG</t>
+          <t>v0: vi phạm loại trừ lẫn nhau tại h6_tranh_chap (CWE-667); v1: đồng bộ mutex đạt chuẩn</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -951,28 +945,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>REQ-15, NFR-04</t>
+          <t>REQ-11, REQ-12</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Worker nhập kho và worker xuất kho tự động cùng đóng phiên</t>
+          <t>H6: Double-free và Use-after-free khi giải phóng phiên kho</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Cụm trạng thái h6_* trong mô hình kết hợp; LoaiTruLanNhau dòng 1 (nhap_locked, xuat_locked)</t>
+          <t>release_stock_items và close_inventory_session - M2 Trang</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Worker xuất kho kích hoạt đúng lúc worker nhập kho đang giữ phiên
-Chạy check_mutual_exclusion(model, 'nhap_locked', 'xuat_locked')</t>
+          <t>Chạy kiểm toán AddressSanitizer trên bản v0 và v1</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>v0: Mutual exclusion VI PHẠM tại h6_tranh_chap (CWE-667); v1: ĐÚNG</t>
+          <t>v0: bắt lỗi use-after-free (CWE-416) và double-free (CWE-415); v1: 0 crash ASan</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -989,109 +982,30 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>REQ-16, REQ-17</t>
+          <t>REQ-01 đến REQ-12</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Double-free và Use-after-free khi giải phóng phiên kho</t>
+          <t>Kiểm chứng toàn luồng quản lý kho hàng kết hợp</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>close_inventory_session (double-free), release_stock_items (use-after-free) - M2 Trang</t>
+          <t>Mô hình kết hợp tổng thể 35 trạng thái</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Gộp mã C của 2 hàm
-Chạy check_c_source()
-Chạy kiểm toán AddressSanitizer</t>
+          <t>Chạy chay_kiem_chung_kripke.py kiểm tra deadlock và 22 công thức CTL</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>v0: double-free (CWE-415) và use-after-free (CWE-416); v1: 0 phát hiện, 0 crash ASan</t>
+          <t>Không deadlock; v0: phát hiện lỗi tại các trạng thái vi phạm; v1: 100% thỏa mãn thuộc tính</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TC-13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>REQ-18, NFR-05, CON-07</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Mã PIN thủ kho còn trong bộ nhớ Heap sau khi giải phóng</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Mô hình con M6 (Đóng phiên kho và thu hồi tài nguyên)</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Nạp M6_dong_phien.json vào tab Ch1
-Chọn luồng M6-v0, kiểm tra AG(!secret_residue)
-Chọn luồng M6-v1, kiểm tra lại</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>M6-v0: VI PHẠM (CWE-226/244, CWE-14); M6-v1 (explicit_bzero trước free): ĐÚNG</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TC-14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>REQ-01 đến REQ-18</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm chứng toàn luồng quản lý kho hàng</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Mô hình kết hợp tổng thể (sheet MoHinhTrangThai 35 trạng thái)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Chạy '1) Sinh Kripke + kiểm chứng (Ch1)'
-Kiểm tra deadlock, AF(flow_end), EF(stock_done), EF(input_rejected)</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Không deadlock; v0: AF(flow_end) và EF(input_rejected) VI PHẠM; v1: tất cả 22 công thức ĐÚNG</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1108,7 +1022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1147,7 +1061,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>H1: Hàm phân tích mã phiếu kho (parse_voucher_id) không được ghi vượt biên bộ đệm Stack 32 byte, kể cả khi mã dài ĐÚNG 32 ký tự (C1.2, C1.3)</t>
+          <t>H1: Hàm nạp chuỗi (ingest_raw_line) không được ghi vượt biên bộ đệm Stack 32 byte, kể cả khi mã dài ĐÚNG 32 ký tự (C1.2, C1.3 - M1 Thọ)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1169,7 +1083,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>H1: Mã phiếu kho hợp lệ không được bị cắt cụt hoặc biến đổi khi lưu vào bộ đệm Stack 32 byte (C1.4)</t>
+          <t>H1: Chuỗi mã phiếu kho hợp lệ (len &lt;= 31 byte) phải được sao chép nguyên vẹn và kết thúc bằng ký tự '\0' (C1.1 - M1 Thọ)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1191,7 +1105,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>H2: Kết quả cấp phát mảng kiện hàng động (create_stock_items) trên Heap phải được kiểm tra NULL trước khi sử dụng (C2.2)</t>
+          <t>H2: Hàm đọc token (get_token_field) phải kiểm tra chỉ số field_idx nằm trong khoảng hợp lệ [0, token_count - 1] trước khi đọc mảng (C2.1, C2.2 - M1 Thọ)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1213,12 +1127,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>H2: Kích thước cấp phát mảng kiện hàng (n * sizeof(Product)) không được gây tràn số nguyên dẫn đến cấp phát thiếu bộ nhớ rồi ghi tràn Heap (C2.3)</t>
+          <t>H2: Con trỏ mảng token_offsets phải được kiểm tra khác NULL và token_count &gt; 0 trước khi đọc phần tử (C2.3 - M1 Thọ)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1235,12 +1149,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>H2: Mọi phần tử kiện hàng trong danh mục động phải được khởi tạo đầy đủ trước khi đọc, không đọc dữ liệu rác (C2.4)</t>
+          <t>H3: Quá trình mở rộng mảng danh mục hàng (expand_stock_items) bằng realloc khi gặp sự cố OOM không được ghi đè làm mất địa chỉ vùng nhớ cũ gây rò rỉ bộ nhớ (C3.1, C3.2 - M2 Trang)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>functional</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1257,12 +1171,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>H3: Phép tính tổng giá trị tiền tồn kho (đơn giá x số lượng + phí đóng gói) không được gây tràn số nguyên có dấu 32-bit (C3.2, C3.3)</t>
+          <t>H3: Kích thước mở rộng mảng động (new_capacity * sizeof(Product)) không được gây tràn số nguyên dẫn đến cấp phát thiếu ô nhớ trên Heap (C3.3 - M2 Trang)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>arithmetic</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1279,12 +1193,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>H3: Giá trị tiền tồn kho không được âm do chiết khấu lớn hơn tạm tính hoặc số lượng âm (C3.4)</t>
+          <t>H4: Phép cộng dồn tồn kho mới vào tồn kho cũ (update_stock_quantity) không được gây tràn số nguyên có dấu 32-bit vượt trần INT_MAX (C4.1, C4.2 - M3 Đô)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1301,17 +1215,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>H3: Phép phân bổ định mức chi phí kho theo kỳ hạn không được chia cho 0 khi kỳ hạn bằng 0 (C3.5)</t>
+          <t>H4: Hệ thống phải từ chối số lượng nhập hàng là số âm (added_quantity &lt;= 0) để đảm bảo toàn vẹn dữ liệu kho (C4.3 - M3 Đô)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>arithmetic</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
     </row>
@@ -1323,12 +1237,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>H4: Chuỗi mã token ủy quyền thủ kho từ nguồn ngoài không được vượt quá 20 ký tự (C4.2)</t>
+          <t>H5: Phép nhân quy đổi giá trị hàng hóa theo tỉ giá (scale_product_price) không được gây tràn số nguyên có dấu 32-bit (C5.1, C5.2 - M3 Đô)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1345,12 +1259,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>H4: Luồng xác thực quyền thủ kho không được chứa nhánh bí mật (magic value) bỏ qua kiểm tra an ninh (C4.3)</t>
+          <t>H6: Hai tiến trình worker nhập kho và worker xuất kho tự động dùng chung phiên kho không được đồng thời can thiệp gây tranh chấp tài nguyên (C6.1 - M2 Trang)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>security</t>
+          <t>concurrency</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1367,12 +1281,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>H4: Phép cộng dồn tồn kho mới vào tồn kho cũ (update_stock_quantity) không được gây tràn số nguyên có dấu 32-bit và phải từ chối số lượng nhập âm (C4.4)</t>
+          <t>H6: Khi đóng phiên kho hàng, con trỏ phiên làm việc không được giải phóng hai lần (CWE-415 Double Free) (C6.2 - M2 Trang)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>arithmetic</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1389,7 +1303,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>H5: Hàm ghi nhật ký kiểm kê kho không được rò rỉ bộ nhớ tiến trình khi tái cấp phát bộ đệm nhật ký (C5.2)</t>
+          <t>H6: Sau khi giải phóng bộ nhớ danh mục hàng hóa (release_stock_items), con trỏ phải được gán NULL ngay lập tức; cấm tuyệt đối đọc/ghi vào vùng nhớ đã giải phóng (CWE-416 Use-After-Free) (C6.3 - M2 Trang)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1398,138 +1312,6 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>REQ-13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>H5: Nội dung ghi nhật ký kiểm kê không được sử dụng trực tiếp chuỗi do người dùng nhập làm format string cho printf/syslog (C5.3)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>security</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>REQ-14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>H5: Phép nhân quy đổi giá trị hàng hóa theo tỉ giá (scale_product_price) không được gây tràn số nguyên có dấu 32-bit (C5.4)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>arithmetic</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>REQ-15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>H6: Hai tiến trình worker nhập kho và worker xuất kho tự động dùng chung phiên kho không được đồng thời can thiệp gây tranh chấp tài nguyên (C6.2)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>concurrency</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>REQ-16</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>H6: Khi đóng phiên kho hàng, con trỏ phiên làm việc không được giải phóng hai lần (CWE-415 Double Free) (C6.3)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>REQ-17</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>H6: Sau khi giải phóng bộ nhớ danh mục hàng hóa (release_stock_items), con trỏ phải được gán NULL ngay lập tức; cấm tuyệt đối đọc/ghi vào vùng nhớ đã giải phóng (CWE-416 Use-After-Free) (C6.4)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>REQ-18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>H6: Bộ nhớ chứa mã PIN thủ kho và dữ liệu nhạy cảm phải được xóa sạch bằng explicit_bzero trước khi gọi free(), không để sót lại trên Heap (C6.5)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>security</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1579,7 +1361,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống xử lý tối thiểu 300 giao dịch xuất nhập kho/giây trên phần cứng máy chủ tham chiếu</t>
+          <t>Hệ thống xử lý tối thiểu 300 giao dịch nạp chuỗi và đọc token/giây trên phần cứng máy chủ tham chiếu</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1596,7 +1378,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Phản hồi xác thực token ủy quyền thủ kho trong tối đa 2 giây (tránh timeout đồng bộ kho phân tán)</t>
+          <t>Phản hồi thao tác kiểm tra biên mảng token trong tối đa 1 mili-giây (thao tác trực tiếp trên RAM)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1647,7 +1429,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Mã PIN thủ kho và token phiên làm việc không tồn tại trong dump bộ nhớ tiến trình sau khi đóng phiên kho</t>
+          <t>Con trỏ mảng động sau khi giải phóng bằng free() phải triệt tiêu hoàn toàn, không để sót dangling pointer</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1684,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1717,7 +1499,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu kho tối đa 31 ký tự ASCII (31 ký tự cần 32 byte bộ đệm Stack kể cả '\0')</t>
+          <t>Chuỗi mã phiếu kho tối đa 31 ký tự ASCII (31 ký tự cần 32 byte bộ đệm Stack kể cả '\0' - M1 Thọ)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1734,7 +1516,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mã token ủy quyền thủ kho tối đa 20 ký tự ASCII (cần 21 byte kể cả '\0')</t>
+          <t>Mảng token_offsets có số phần tử token_count &gt; 0; chỉ số đọc field_idx phải thỏa 0 &lt;= field_idx &lt; token_count (M1 Thọ)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1751,7 +1533,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mỗi phiếu có 1–100 dòng kiện hàng; số lượng mỗi dòng 1–1000; đơn giá 0–50.000.000 VND; giá trị mỗi dòng tối đa 50.000.000 VND</t>
+          <t>Danh mục hàng hóa khởi tạo ban đầu có dung lượng 16 phần tử; khi đầy nhân đôi thành 32 phần tử trên Heap (M2 Trang)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1768,7 +1550,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Đơn giá và tổng tiền là số nguyên có dấu 32-bit (signed int, đơn vị VND)</t>
+          <t>Số lượng tồn kho, số lượng nhập thêm và đơn giá là số nguyên có dấu 32-bit (signed int, tối đa INT_MAX = 2.147.483.647 - M3 Đô)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1785,12 +1567,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Số kỳ hạn phân bổ định mức chi phí kho từ 1 đến 24 tháng</t>
+          <t>Worker quét xuất kho tự động kích hoạt định kỳ sau 15 phút rảnh phiên (M2 Trang)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
@@ -1802,27 +1584,10 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Worker quét xuất kho tự động kích hoạt định kỳ sau 15 phút rảnh phiên</t>
+          <t>Mảng động danh mục hàng ProductList bắt buộc cấp phát trên Heap qua malloc/realloc và giải phóng qua free (M2 Trang)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>CON-07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Bộ nhớ chứa mã PIN thủ kho và mảng kiện hàng động bắt buộc cấp phát trên Heap qua malloc/calloc</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1839,13 +1604,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1938,7 +1703,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nhận chuỗi mã phiếu kho từ giao diện</t>
+          <t>Nhận chuỗi mã phiếu kho vào bộ đệm stack 32 byte (M1 Thọ)</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1731,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu chép đủ vào buffer 32 byte, có '\0' (an toàn)</t>
+          <t>Chuỗi mã phiếu &lt;= 31 byte chép thành công có '\0' (an toàn)</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1759,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu dài đúng 32 ký tự: ghi đè byte '\0' vào byte lân cận (lỗi ẩn Off-by-one)</t>
+          <t>Chuỗi dài đúng 32 ký tự: ghi đè byte '\0' ra ngoài bộ đệm (CWE-193 Off-by-one)</t>
         </is>
       </c>
     </row>
@@ -2022,7 +1787,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mã phiếu dài &gt; 32 byte: ghi đè tràn stack frame (lỗi hiện Buffer Overflow)</t>
+          <t>Chuỗi dài &gt;= 33 byte: ghi đè tràn stack frame (CWE-120/121 Buffer Overflow)</t>
         </is>
       </c>
     </row>
@@ -2035,12 +1800,12 @@
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>h2, allocating</t>
+          <t>h2, indexing</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>h2_ok, h2_null, h2_sai_kich_thuoc, h2_doc_rac</t>
+          <t>h2_ok, h2_doc_ngoai_bien, h2_chi_so_am, h2_null_mang</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -2050,7 +1815,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>items = malloc(n * sizeof(Product))</t>
+          <t>Đọc trường dữ liệu token theo chỉ số mảng (M1 Thọ)</t>
         </is>
       </c>
     </row>
@@ -2063,7 +1828,7 @@
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>h2, allocated, initialized</t>
+          <t>h2, index_ok, read_ok</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2078,20 +1843,20 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Cấp phát thành công và đã khởi tạo struct (an toàn)</t>
+          <t>Chỉ số 0 &lt;= field_idx &lt; token_count: đọc token thành công (an toàn)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>h2_null</t>
+          <t>h2_doc_ngoai_bien</t>
         </is>
       </c>
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>h2, null_deref, violation</t>
+          <t>h2, out_of_bounds_read, violation</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2106,20 +1871,20 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>malloc trả NULL khi hết RAM nhưng vẫn truy cập ghi vào (lỗi ẩn OOM)</t>
+          <t>Chỉ số field_idx &gt;= token_count: đọc ngoài biên trên mảng (CWE-125)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>h2_sai_kich_thuoc</t>
+          <t>h2_chi_so_am</t>
         </is>
       </c>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>h2, alloc_size_overflow, heap_overflow, violation</t>
+          <t>h2, out_of_bounds_read, violation</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -2134,20 +1899,20 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>n*48 tràn int32 hoặc n âm: cấp phát sai kích thước rồi ghi tràn Heap (lỗi ẩn)</t>
+          <t>Chỉ số field_idx &lt; 0: đọc ngược vùng nhớ trước mảng (CWE-125)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>h2_doc_rac</t>
+          <t>h2_null_mang</t>
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>h2, uninit_read, violation</t>
+          <t>h2, null_deref, violation</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2162,7 +1927,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Đọc dữ liệu kiện hàng khi chưa khởi tạo memset/calloc (lỗi ẩn Uninit Read)</t>
+          <t>Mảng token_offsets == NULL hoặc token_count &lt;= 0 (CWE-476 NULL Deref)</t>
         </is>
       </c>
     </row>
@@ -2175,12 +1940,12 @@
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>h3, computing</t>
+          <t>h3, allocating</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>h3_ok, h3_tran_so, h3_so_am, h3_chia_0</t>
+          <t>h3_ok, h3_ro_ri_oom, h3_tran_kich_thuoc</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2190,7 +1955,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Tính tổng tồn kho = Σ đơn giá × SL + phí đóng gói − chiết khấu</t>
+          <t>Mở rộng mảng danh mục hàng khi danh sách đầy bằng realloc (M2 Trang)</t>
         </is>
       </c>
     </row>
@@ -2203,7 +1968,7 @@
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>h3, amount_ok</t>
+          <t>h3, realloc_ok</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -2218,20 +1983,20 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Tổng giá trị tồn kho nằm trong miền hợp lệ [0, 2 tỷ VND] (an toàn)</t>
+          <t>Tái cấp phát thành công, nhân đôi dung lượng an toàn</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>h3_tran_so</t>
+          <t>h3_ro_ri_oom</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>h3, int_overflow, violation</t>
+          <t>h3, mem_leak, violation</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2241,25 +2006,25 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>C3.2/C3.3</t>
+          <t>C3.2</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Tràn int32 khi nhân đơn giá x SL hoặc khi cộng dồn nhiều kiện (lỗi ẩn)</t>
+          <t>realloc trả về NULL, con trỏ gốc bị ghi đè gây mất mảng cũ (CWE-401 Memory Leak)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>h3_so_am</t>
+          <t>h3_tran_kich_thuoc</t>
         </is>
       </c>
       <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>h3, negative_amount, violation</t>
+          <t>h3, alloc_size_overflow, violation</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2269,109 +2034,109 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>C3.4</t>
+          <t>C3.3</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>SL/chiết khấu âm hoặc chiết khấu &gt; tạm tính: tổng tiền âm (lỗi ẩn)</t>
+          <t>new_capacity * sizeof(Product) tràn int32 dẫn tới cấp phát thiếu Heap</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>h3_chia_0</t>
+          <t>h4_vao</t>
         </is>
       </c>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>h3, div_by_zero, violation</t>
+          <t>h4, computing</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>dung_khong_an_toan</t>
+          <t>h4_ok, h4_tran_so_am, h4_so_luong_am</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>C3.5</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Phân bổ chiết khấu với kỳ hạn = 0: chia cho 0 gây crash tiến trình</t>
+          <t>Cộng dồn số lượng tồn kho mới vào tồn kho cũ (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>h4_vao</t>
+          <t>h4_ok</t>
         </is>
       </c>
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>h4, validating</t>
+          <t>h4, sum_ok</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>h4_ok, h4_tran_token, h4_nhanh_an, h4_tu_choi_quyen</t>
+          <t>h5_vao</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>C4.1</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Xác thực token ủy quyền thủ kho và cộng dồn số lượng tồn kho</t>
+          <t>current_stock + added_quantity &lt;= INT_MAX: cộng dồn an toàn</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>h4_ok</t>
+          <t>h4_tran_so_am</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>h4, token_ok, authorized</t>
+          <t>h4, int_overflow, violation</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>h5_vao</t>
+          <t>dung_khong_an_toan</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>C4.1</t>
+          <t>C4.2</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Token hợp lệ, chữ ký đúng, cập nhật tồn kho an toàn</t>
+          <t>current_stock + added_quantity vượt 2^31 - 1: tràn số nguyên lật âm (CWE-190)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>h4_tran_token</t>
+          <t>h4_so_luong_am</t>
         </is>
       </c>
       <c r="B19" s="2" t="n"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>h4, stack_buffer_overflow, violation</t>
+          <t>h4, negative_amount, violation</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2381,53 +2146,53 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>C4.2</t>
+          <t>C4.3</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Token ủy quyền dài &gt; 20 byte: ghi tràn bộ đệm token (lỗi hiện)</t>
+          <t>added_quantity &lt; 0: số lượng nhập âm làm sai lệch kho hàng</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>h4_nhanh_an</t>
+          <t>h5_vao</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>h4, hidden_bypass, violation</t>
+          <t>h5, scaling</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>dung_khong_an_toan</t>
+          <t>h5_ok, h5_nhan_tran_int</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>C4.3</t>
+          <t>H5</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Token mang giá trị ma thuật (magic value 31337/8080) bỏ qua xác thực (cửa sau ẩn)</t>
+          <t>Quy đổi đơn giá sản phẩm theo tỉ giá (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>h4_tu_choi_quyen</t>
+          <t>h5_ok</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>h4, token_invalid</t>
+          <t>h5, scale_ok</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2437,249 +2202,249 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>C4.4</t>
+          <t>C5.1</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Token sai: từ chối quyền nhưng vẫn đẩy phiên sang bước đóng (an toàn)</t>
+          <t>base_price * rate &lt;= INT_MAX: nhân tỉ giá an toàn</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>h5_vao</t>
+          <t>h5_nhan_tran_int</t>
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>h5, logging</t>
+          <t>h5, int_overflow, violation</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>h5_ok, h5_ro_ri, h5_format_string</t>
+          <t>dung_khong_an_toan</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>H5</t>
+          <t>C5.2</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Ghi nhật ký kiểm kê kho và quy đổi đơn giá sản phẩm</t>
+          <t>base_price * rate vượt INT_MAX: tràn phép nhân số nguyên (CWE-190)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>h5_ok</t>
+          <t>h6_phien_ranh</t>
         </is>
       </c>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>h5, log_ok, audit_clean</t>
+          <t>h6, sess_free</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>h6_phien_ranh</t>
+          <t>h6_nhap_giu, h6_xuat_giu</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>C5.1</t>
+          <t>H6</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Ghi log thành công, giải phóng bộ đệm log sạch sẽ</t>
+          <t>Phiên kho rảnh, chờ worker kết thúc phiên (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>h5_ro_ri</t>
+          <t>h6_nhap_giu</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>h5, mem_leak, violation</t>
+          <t>h6, nhap_locked</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>dung_khong_an_toan</t>
+          <t>h6_giai_phong, h6_tranh_chap</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>C5.2</t>
+          <t>C6.1</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>realloc bộ đệm log thất bại gán đè NULL làm mất con trỏ cũ (CWE-401 rò rỉ bộ nhớ)</t>
+          <t>Worker nhập kho giữ khóa phiên làm việc</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>h5_format_string</t>
+          <t>h6_xuat_giu</t>
         </is>
       </c>
       <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>h5, format_string, violation</t>
+          <t>h6, xuat_locked</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>dung_khong_an_toan</t>
+          <t>h6_giai_phong, h6_tranh_chap</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>C5.3</t>
+          <t>C6.1</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>syslog(LOG_INFO, raw_comment): chuỗi nhập chứa %x/%n đọc ghi tùy ý bộ nhớ</t>
+          <t>Worker xuất kho tự động giữ khóa phiên</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>h6_phien_ranh</t>
+          <t>h6_tranh_chap</t>
         </is>
       </c>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>h6, sess_free</t>
+          <t>h6, nhap_locked, xuat_locked, race, violation</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>h6_nhap_giu, h6_xuat_giu</t>
+          <t>h6_double_free, h6_uaf</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>H6</t>
+          <t>C6.2</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Phiên kho đang mở, chưa worker nào giữ khóa</t>
+          <t>Cả 2 worker cùng giữ phiên (Race condition vi phạm loại trừ lẫn nhau)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>h6_nhap_giu</t>
+          <t>h6_double_free</t>
         </is>
       </c>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>h6, nhap_locked</t>
+          <t>h6, double_free, violation</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>h6_giai_phong, h6_tranh_chap</t>
+          <t>dung_khong_an_toan</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>C6.1</t>
+          <t>C6.3</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Worker nhập kho đang giữ khóa phiên làm việc</t>
+          <t>Cả 2 worker cùng gọi free() trên cùng con trỏ phiên (CWE-415)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>h6_xuat_giu</t>
+          <t>h6_uaf</t>
         </is>
       </c>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>h6, xuat_locked</t>
+          <t>h6, use_after_free, violation</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>h6_giai_phong, h6_tranh_chap</t>
+          <t>dung_khong_an_toan</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>C6.1</t>
+          <t>C6.4</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Worker xuất kho tự động (15 phút) đang giữ khóa phiên</t>
+          <t>Worker đến sau đọc/ghi vào vùng nhớ phiên đã bị free (CWE-416)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>h6_tranh_chap</t>
+          <t>h6_giai_phong</t>
         </is>
       </c>
       <c r="B29" s="2" t="n"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>h6, nhap_locked, xuat_locked, race, violation</t>
+          <t>h6, releasing</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>h6_double_free, h6_uaf</t>
+          <t>ket_thuc_ok, h6_uaf_dangling</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>C6.2</t>
+          <t>C6.1</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Cả 2 worker cùng giữ phiên (Race condition, vi phạm loại trừ lẫn nhau)</t>
+          <t>Giải phóng tài nguyên danh mục hàng hóa</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>h6_double_free</t>
+          <t>h6_uaf_dangling</t>
         </is>
       </c>
       <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>h6, double_free, violation</t>
+          <t>h6, use_after_free, violation</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2689,81 +2454,81 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>C6.3</t>
+          <t>C6.5</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Cả 2 worker cùng gọi free(session) trên cùng một con trỏ (CWE-415)</t>
+          <t>Sau free(items) không gán NULL, đọc lại items[0] gây Use-After-Free (CWE-416)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>h6_uaf</t>
+          <t>ket_thuc_ok</t>
         </is>
       </c>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>h6, use_after_free, violation</t>
+          <t>flow_end, stock_done, mem_clean, safe</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>dung_khong_an_toan</t>
+          <t>ket_thuc_ok</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>C6.4</t>
+          <t>C6.1</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Worker đến sau đọc/ghi vào phiên kho đã bị worker trước free (CWE-416)</t>
+          <t>Phiên kho kết thúc thành công, giải phóng toàn bộ bộ nhớ (trạng thái an toàn)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>h6_giai_phong</t>
+          <t>ket_thuc_tu_choi</t>
         </is>
       </c>
       <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>h6, releasing</t>
+          <t>flow_end, input_rejected, mem_clean, safe</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ket_thuc_ok, h6_con_ma_pin</t>
+          <t>ket_thuc_tu_choi</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>C6.1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Giải phóng bộ đệm mã PIN thủ kho và mảng sản phẩm</t>
+          <t>Từ chối dữ liệu đầu vào không hợp lệ có kiểm soát (v0 thiếu nhánh này)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>h6_con_ma_pin</t>
+          <t>dung_khong_an_toan</t>
         </is>
       </c>
       <c r="B33" s="2" t="n"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>h6, secret_residue, violation</t>
+          <t>flow_end, unsafe_halt, violation</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2773,96 +2538,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>C6.5</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Mã PIN thủ kho còn nguyên trong Heap sau free (memset bị compiler tối ưu -O2 loại bỏ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>ket_thuc_ok</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>flow_end, stock_done, mem_clean, safe</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>ket_thuc_ok</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>C6.1</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Phiên kho kết thúc thành công, giải phóng toàn bộ bộ nhớ (trạng thái an toàn)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>ket_thuc_tu_choi</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>flow_end, input_rejected, mem_clean, safe</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>ket_thuc_tu_choi</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>C1.4/C4.4</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Từ chối đầu vào không hợp lệ, thu hồi bộ nhớ an toàn (v0 thiếu nhánh này)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>dung_khong_an_toan</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>flow_end, unsafe_halt, violation</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>dung_khong_an_toan</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Tiến trình sập (crash SIGSEGV/ABORT) do vi phạm an toàn bộ nhớ</t>
+          <t>Tiến trình crash (SIGSEGV/ABORT) do vi phạm an toàn bộ nhớ</t>
         </is>
       </c>
     </row>
@@ -2877,10 +2558,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2911,12 +2592,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AG(!buffer_overflow)</t>
+          <t>AG(!stack_buffer_overflow)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Safety C1.2, C1.3, C4.2 — CWE-120/787 (tràn stack bộ đệm mã phiếu 32 byte và token 20 byte)</t>
+          <t>Safety H1 — CWE-120/121 (tràn stack bộ đệm mã phiếu 32 byte - M1 Thọ)</t>
         </is>
       </c>
     </row>
@@ -2928,233 +2609,185 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Safety C1.2 — CWE-193 (lỗi ẩn: mã phiếu dài đúng 32 ký tự ghi đè null terminator)</t>
+          <t>Safety H1 — CWE-193 (mã phiếu dài đúng 32 ký tự ghi đè byte null - M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AG(!null_deref)</t>
+          <t>AG(!out_of_bounds_read)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Safety C2.2 — CWE-476 (lỗi ẩn: malloc trả NULL khi cạn RAM nhưng vẫn ghi vào)</t>
+          <t>Safety H2 — CWE-125 (đọc token ngoài biên mảng hoặc chỉ số âm - M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AG(!alloc_size_overflow)</t>
+          <t>AG(!null_deref)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Safety C2.3 — CWE-190/787 (lỗi ẩn: n * 48 byte tràn int32 dẫn tới cấp phát thiếu ô nhớ trên Heap)</t>
+          <t>Safety H2 — CWE-476 (đọc mảng token khi con trỏ NULL - M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AG(!uninit_read)</t>
+          <t>AG(!alloc_size_overflow)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Safety C2.4 — CWE-457 (lỗi ẩn: đọc trường trạng thái kiện hàng khi chưa khởi tạo)</t>
+          <t>Safety H3 — CWE-190/787 (kích thước mở rộng mảng n * 48 byte tràn int32 - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AG(!int_overflow)</t>
+          <t>AG(!mem_leak)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Safety C3.2, C3.3, C4.4 — CWE-190 (lỗi ẩn: nhân đơn giá tràn int32 hoặc cộng dồn tồn kho vượt 2 tỷ)</t>
+          <t>Safety H3 — CWE-401 (realloc mở rộng mảng khi OOM làm mất con trỏ cũ - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AG(!negative_amount)</t>
+          <t>AG(!int_overflow)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Safety C3.4, C4.4 (lỗi ẩn: số lượng âm hoặc chiết khấu lớn hơn tạm tính làm tổng âm)</t>
+          <t>Safety H4, H5 — CWE-190 (cộng dồn tồn kho vượt 2 tỷ hoặc nhân tỉ giá tràn int32 - M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AG(!div_by_zero)</t>
+          <t>AG(!negative_amount)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Safety C3.5 — CWE-369 (lỗi crash: phân bổ chi phí kho với kỳ hạn bằng 0)</t>
+          <t>Safety H4 — (số lượng nhập hàng là số âm làm sai lệch số liệu kho - M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AG(!hidden_bypass)</t>
+          <t>AG(!race)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Safety C4.3 — CWE-912 (lỗi ẩn: token ma thuật 31337/8080 vượt mặt xác thực thủ kho)</t>
+          <t>Safety H6 — CWE-667 (worker nhập kho và worker xuất kho tự động cùng chiếm phiên - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AG(!mem_leak)</t>
+          <t>AG(!double_free)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Safety C5.2 — CWE-401 (lỗi ẩn: realloc thất bại gán đè NULL làm rò rỉ vùng nhớ tiến trình)</t>
+          <t>Safety H6 — CWE-415 (giải phóng phiên kho 2 lần liên tiếp - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AG(!format_string)</t>
+          <t>AG(!use_after_free)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Safety C5.3 — CWE-134 (lỗi bảo mật: chuỗi format string trong ghi nhật ký kiểm kê)</t>
+          <t>Safety H6 — CWE-416 (đọc dữ liệu con trỏ treo sau khi free - M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>AG(!race)</t>
+          <t>AF(flow_end)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.2 — CWE-667 (lỗi ẩn: worker nhập kho và worker xuất kho tự động cùng chiếm phiên)</t>
+          <t>Liveness: mọi nhánh xử lý đều kết thúc có kiểm soát</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>AG(!double_free)</t>
+          <t>EF(stock_done)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.3 — CWE-415 (lỗi crash: giải phóng phiên kho 2 lần liên tiếp)</t>
+          <t>Khả đạt: tồn tại đường đi hoàn thành phiên kho an toàn thành công</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>AG(!use_after_free)</t>
+          <t>EF(input_rejected)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.4 — CWE-416 (lỗi ẩn: đọc/ghi dữ liệu sau khi đã gọi free phiên kho)</t>
+          <t>Khả đạt: tồn tại nhánh từ chối đầu vào độc hại/sai cú pháp (v0 KHÔNG có -&gt; VI PHẠM)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>AG(!secret_residue)</t>
+          <t>EG(!violation)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Safety C6.5 — CWE-226/14 (lỗi ẩn: mã PIN thủ kho còn sót lại trên Heap sau khi giải phóng)</t>
+          <t>Tồn tại ít nhất một đường đi luôn an toàn từ đầu đến cuối</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AF(flow_end)</t>
+          <t>EF(nhap_locked)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Liveness: mọi nhánh xử lý đều kết thúc (v0 kẹt tại trạng thái vi phạm lặp vô tận)</t>
+          <t>Khả đạt của cụm khóa phiên nhập kho (mô hình khóa phiên hoạt động được)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EF(stock_done)</t>
+          <t>EF(xuat_locked)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Khả đạt REQ-18: tồn tại đường đi hoàn thành phiên kho an toàn thành công</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>EF(input_rejected)</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Khả đạt: tồn tại nhánh từ chối đầu vào độc hại/sai cú pháp (v0 KHÔNG có -&gt; VI PHẠM)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>EG(!violation)</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Tồn tại ít nhất một đường đi luôn an toàn từ đầu đến cuối</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>EF(nhap_locked)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Khả đạt của cụm khóa phiên nhập kho (mô hình khóa phiên hoạt động được)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>EF(xuat_locked)</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Khả đạt của cụm khóa phiên xuất kho tự động (mô hình khóa phiên hoạt động được)</t>
         </is>
@@ -3171,7 +2804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -3245,18 +2878,6 @@
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>mem_clean</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>secret_residue</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>mem_clean</t>
         </is>
@@ -3273,18 +2894,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="64" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3337,7 +2958,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>parse_voucher_id</t>
+          <t>ingest_raw_line</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3352,7 +2973,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>raw_voucher_id</t>
+          <t>dst, cap, raw_line</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -3367,14 +2988,14 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>H1 — C1.2/C1.3 (CON-01 bộ đệm Stack 32 byte - M1 Thọ)</t>
+          <t>H1 — Nạp chuỗi vào bộ đệm stack 32 byte (M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>parse_auth_token</t>
+          <t>get_token_field</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -3384,34 +3005,32 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>buffer_copy</t>
+          <t>array_read</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>raw_token</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>20</v>
-      </c>
+          <t>token_offsets, token_count, field_idx</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>buffer-overflow</t>
+          <t>out-of-bounds-read</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>H4 — C4.2 (CON-02 token 20 byte)</t>
+          <t>H2 — Đọc trường token theo chỉ số mảng (M1 Thọ)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>create_stock_items</t>
+          <t>expand_stock_items</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3424,23 +3043,31 @@
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>list, new_capacity</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F4" s="2" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>memory-leak</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>H2 — C2.2/C2.3/C2.4 cấp phát động struct Product trên Heap (M2 Trang)</t>
+          <t>H3 — realloc mở rộng mảng khi OOM gây rò rỉ bộ nhớ (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>expand_stock_items</t>
+          <t>release_stock_items</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -3453,27 +3080,31 @@
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>list</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="n">
         <v>16</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>memory-leak</t>
+          <t>use-after-free</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>H3 — realloc mảng động khi OOM làm mất con trỏ gốc (CWE-401 - M2 Trang)</t>
+          <t>H6 — free() không gán NULL dẫn tới Use-After-Free (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>release_stock_items</t>
+          <t>update_stock_quantity</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3483,30 +3114,32 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>alloc_release</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n">
-        <v>16</v>
-      </c>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>current_stock, added_quantity</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>use-after-free</t>
+          <t>integer-overflow</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>H6 — free() không gán NULL dẫn tới Use-After-Free (CWE-416 - M2 Trang)</t>
+          <t>H4 — Cộng dồn tồn kho tràn signed int 32-bit (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>write_inventory_log</t>
+          <t>scale_product_price</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -3516,184 +3149,60 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>alloc_release</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n">
-        <v>32</v>
-      </c>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>base_price, rate</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>memory-leak</t>
+          <t>integer-overflow</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>H5 — C5.2 rò rỉ bộ nhớ khi mở rộng buffer log</t>
+          <t>H5 — Nhân tỉ giá quy đổi tràn int32 (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>close_inventory_session</t>
+          <t>calc_batch_capacity</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>python</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>alloc_release</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n">
-        <v>4</v>
-      </c>
+          <t>divide</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>total_items, batch_size</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>double-free</t>
+          <t>divide-by-zero</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>H6 — C6.3 giải phóng phiên làm việc hai lần (CWE-415)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>update_stock_quantity</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>arithmetic</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>current_stock, added_quantity</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>H4 — C4.4 cộng dồn tồn kho tràn signed int 32-bit (M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>scale_product_price</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>arithmetic</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>base_price, rate</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>H5 — C5.4 nhân tỉ giá quy đổi tràn int32 (M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>calc_batch_capacity</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>divide</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>total_items, batch_size</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>H3 — C3.5 chia cho 0 khi batch_size = 0 (black-box fuzz)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>auth_debug_bypass</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>magic_value</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>warehouse_id, debug_pin</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n">
-        <v>31337</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>8080</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>H4 — C4.3 nhánh ẩn backdoor vượt mặt xác thực (concolic)</t>
+          <t>H3 — Chia cho 0 khi batch_size = 0 (black-box fuzz)</t>
         </is>
       </c>
     </row>
@@ -3708,10 +3217,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
@@ -3768,7 +3277,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>C4.4 — phép cộng dồn tồn kho mới vào tồn kho cũ vượt trần INT_MAX (M3 Đô)</t>
+          <t>H4 — phép cộng dồn tồn kho mới vào tồn kho cũ vượt trần INT_MAX (M3 Đô)</t>
         </is>
       </c>
     </row>
@@ -3795,115 +3304,61 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C2.3 — kích thước tái cấp phát Heap vượt 2GB khi new_capacity lớn (M2 Trang)</t>
+          <t>H3 — kích thước tái cấp phát Heap vượt 2GB khi new_capacity lớn (M2 Trang)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>line_amount_mul</t>
+          <t>price_multiplication_overflow</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>price, qty</t>
+          <t>base_price, rate</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>price &gt;= 0 and price &lt;= 50000000 and qty &gt;= 1 and qty &lt;= 1000 and price * qty &gt; 2147483647</t>
+          <t>base_price &gt; 0 and rate &gt; 1 and base_price * rate &gt; 2147483647</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>price * qty</t>
+          <t>base_price * rate</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>C3.2 — phép nhân đơn giá x số lượng tràn TRƯỚC khi kịp kiểm tra hạn mức dòng</t>
+          <t>H5 — phép nhân đơn giá x tỉ giá quy đổi tràn int32 (M3 Đô)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>accumulated_total</t>
+          <t>negative_quantity_check</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>total_before, line_total</t>
+          <t>added_quantity</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>total_before &gt;= 0 and total_before &lt;= 2147483647 and line_total &gt;= 0 and line_total &lt;= 50000000 and total_before + line_total &gt; 2147483647</t>
+          <t>added_quantity &lt; 0</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>total_before + line_total</t>
+          <t>added_quantity</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>C3.3 — bước cộng dồn nhiều kiện hàng: mỗi kiện hợp lệ nhưng tổng vượt trần int32</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>negative_quantity_check</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity &lt; 0</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>C4.4 — số lượng nhập hàng là số âm làm sai lệch số liệu kho (M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>negative_total</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>subtotal, discount</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>subtotal &gt;= 0 and subtotal &lt;= 2000000000 and discount + 2000000000 &gt;= 0 and discount &lt;= 2000000000 and subtotal - discount &lt; 0</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>subtotal - discount</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>C3.4 — chiết khấu giảm giá âm hoặc lớn hơn tạm tính làm tổng tiền âm</t>
+          <t>H4 — số lượng nhập hàng là số âm làm sai lệch số liệu kho (M3 Đô)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cap nhat quanly_khohang_v0.xlsx: dong bo 7 ham sinh ma, 6 phep z3 va 28 test cases
</commit_message>
<xml_diff>
--- a/01_spec/quanly_khohang_v0.xlsx
+++ b/01_spec/quanly_khohang_v0.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -562,450 +562,1060 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>TC-01</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>REQ-01, CON-01</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>H1: Nạp chuỗi đúng 32 byte gây lỗi Off-by-one và 33 byte tràn stack</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>ingest_raw_line sinh từ đặc tả (v0: buffer 32 byte, Loi=buffer-overflow) - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Gọi ingest_raw_line_v0 với chuỗi 32 và 33 ký tự
-Chạy kiểm tra AG(!stack_buffer_overflow), AG(!off_by_one)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>v0: ghi đè byte '\0' và tràn stack frame (CWE-120/121, CWE-193); v1: rào chắn từ chối trả về -2</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC-M1-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Nạp dòng chuỗi chuẩn độ dài ngắn (len = 15 &lt; 32 bytes) vào buffer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chuỗi raw_line hợp lệ: SP001;GaoST25;100;25000 (23 bytes)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Khởi tạo buffer stack 32 byte
+Thực hiện nạp chuỗi raw_line vào buffer</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>v0 và v1 đều nạp chuỗi thành công, buffer nhận đúng nội dung</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>TC-02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>REQ-02, CON-01</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>H1: Nạp chuỗi hợp lệ 31 byte vào bộ đệm stack 32 byte</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>char buffer[32], cap = 32, chuỗi đầu vào dài đúng 31 ký tự - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Gọi v0 và v1 với chuỗi 31 byte
-Kiểm tra giá trị trả về và nội dung bộ đệm</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Cả 2 phiên bản trả về 31, sao chép thành công có '\0'</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC-M1-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nạp dòng chuỗi cận trên an toàn (len = 31 bytes có null-terminator)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Chuỗi raw_line dài chính xác 31 ký tự + 1 byte null = 32 byte</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Khởi tạo buffer stack 32 byte
+Nạp chuỗi biên 31 byte vào buffer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>v0 và v1 đều sao chép an toàn, ký tự kết thúc chuỗi '\0' được bảo toàn</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TC-03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>REQ-03, CON-02</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>H2: Đọc token tại chỉ số chạm biên trên field_idx == token_count</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>token_offsets có 4 phần tử (chỉ số 0..3), field_idx = 4 - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Gọi get_token_field_v0 với field_idx = 4 dưới giám sát ASan
-Gọi get_token_field_v1 với cùng tham số</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>v0: Đọc ngoài biên mảng token (CWE-125); v1: Rào chắn chặn trả về -2</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC-M1-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>REQ-2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Đọc trường token đầu tiên (field_idx = 0) từ danh sách token hợp lệ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mảng token đã phân tách gồm 4 trường SP001, GaoST25, 100, 25000 (token_count = 4)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gọi hàm get_token_field với field_idx = 0
+Lấy giá trị mã hàng</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Truy xuất thành công trường mã hàng SP001, không lỗi</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TC-04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>REQ-04, CON-02</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>H2: Đọc token với chỉ số âm field_idx &lt; 0</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>token_count = 4, field_idx = -1 - M1 Thọ</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Gọi get_token_field_v0 với field_idx = -1
-Gọi đối chứng get_token_field_v1</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>v0: Đọc lùi vùng nhớ trước mảng (CWE-125); v1: Từ chối an toàn trả về -2</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC-M1-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>REQ-2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Đọc trường token cuối cùng (field_idx = token_count - 1)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>token_count = 4, truy xuất trường đơn giá tại chỉ số 3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gọi hàm get_token_field với field_idx = 3
+Lấy giá trị đơn giá</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Truy xuất thành công trường đơn giá 25000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TC-05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>REQ-05, CON-03</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>H3: Mô phỏng sự cố OOM khi realloc mảng danh mục hàng</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>realloc trả về NULL khi hệ thống cạn kiệt RAM - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Gọi expand_stock_items trên bản v0 và v1 khi mảng đầy cần nhân đôi
-Quan sát con trỏ list</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>v0: list bị gán NULL làm mất địa chỉ mảng cũ (CWE-401 Leak); v1: giữ nguyên con trỏ cũ qua biến tạm tmp</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC-M1-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>REQ-3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kiểm toán an toàn chu trình I/O toàn diện không vi phạm bộ nhớ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Chạy qua toàn bộ chu trình nạp chuỗi và đọc token</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kiểm tra bất biến AG(!violation) trên toàn bộ không gian trạng thái</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>v0: Vi phạm an toàn (CWE-120/125); v1: Thỏa mãn 100% AG(!violation)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC-06</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>REQ-06, CON-03</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>H3: Tràn số nguyên khi tính toán kích thước mở rộng mảng động</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity lớn gây tràn phép nhân new_capacity * sizeof(Product) - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC-M1-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kích hoạt lỗi tràn bộ đệm stack với chuỗi dữ liệu vượt ngưỡng (len = 64 bytes)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Chuỗi raw_line chứa 64 ký tự (vượt quá stack buffer 32 byte)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Gọi ingest_raw_line với chuỗi 64 byte
+Quan sát vùng nhớ stack liền kề</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>v0: Ghi đè frame stack và con trỏ trả về (CWE-120/121); v1: Chặn từ chối an toàn do len &gt;= 32</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC-M1-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bắt lỗi Off-by-one khi chuỗi có đúng 32 byte dữ liệu thiếu null-terminator</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Chuỗi đầu vào có đúng 32 ký tự, không còn chỗ cho ký tự null kết thúc chuỗi</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sao chép 32 byte vào buffer[32] bằng strcpy
+Đọc chuỗi sau khi sao chép</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>v0: Đọc tràn qua biến tiếp theo trên stack do thiếu null (CWE-193); v1: buffer[31] = '\0'</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-M1-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Phát hiện lỗi Stack Buffer Overflow bằng AddressSanitizer (ASan Crash Trigger)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Biên dịch mã nguồn C với flag -fsanitize=address</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Thực thi hàm ingest_raw_line với chuỗi 48 ký tự
+Ghi nhận cảnh báo từ ASan</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>v0: ASan báo lỗi ERROR: AddressSanitizer: stack-buffer-overflow; v1: 0 crash</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-M1-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bắt lỗi đọc ngoài biên mảng token khi chỉ số vượt trần (field_idx &gt;= token_count)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>token_count = 4, yêu cầu đọc trường tại field_idx = 4 hoặc field_idx = 10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Gọi get_token_field(4, 4)
+Kiểm tra con trỏ token trả về</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>v0: Đọc ngoài biên mảng con trỏ token (CWE-125); v1: Phát hiện và trả về NULL/mã lỗi an toàn</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-M1-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Bắt lỗi đọc ngoài biên mảng token khi chỉ số âm (field_idx = -1 &lt; 0)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Yêu cầu đọc trường với chỉ số âm field_idx = -1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Gọi get_token_field(4, -1)
+Kiểm tra phản hồi của hệ thống</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>v0: Đọc vùng nhớ phía trước mảng token (CWE-125); v1: Chặn ngay tại điều kiện field_idx &lt; 0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-M1-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>REQ-6</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kiểm tra tính sống: Không xảy ra deadlock trong toàn bộ chu trình xử lý I/O</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mô hình chuyển trạng thái Kripke của module M1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Duyệt qua tất cả 7 trạng thái
+Kiểm tra bậc ra out-degree của từng trạng thái</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mọi trạng thái đều có out-degree &gt;= 1, 0 deadlock, công thức AF(done) thỏa mãn trên v1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-M1-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-2, REQ-3, REQ-4, REQ-5, REQ-6</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kiểm thử hồi quy đối chứng toàn diện pytest (Regression Verification Suite)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bộ test pytest tự động test_verify_v0_cases_on_v1.py</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Chạy kiểm thử toàn bộ test cases trên bản v0
+Chạy kiểm thử toàn bộ test cases trên bản v1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>v0: Bắt đầy đủ lỗi CWE-120/121, CWE-193, CWE-125; v1: 100% PASSED</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-M2-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Khởi tạo mảng động danh mục hàng ban đầu (Initial Capacity)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Khởi tạo danh sách rỗng product_list_init(&amp;list)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gọi hàm khởi tạo danh mục
+Kiểm tra count == 0, capacity == 16, con trỏ items != NULL</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Thành công: Cấp phát đúng 16 ô nhớ ban đầu trên Heap</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-M2-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>REQ-1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Thêm sản phẩm tới chạm ngưỡng dung lượng chưa mở rộng (Fill to Capacity)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Danh sách đang có capacity = 16</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Thêm liên tiếp 16 sản phẩm hợp lệ vào danh sách
+Kiểm tra count == 16, capacity == 16</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Thành công: 16 sản phẩm được lưu trọn vẹn, chưa kích hoạt realloc</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-M2-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-6</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tự động nhân đôi dung lượng khi thêm sản phẩm thứ 17 (Capacity Doubling)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Danh sách đã đầy 16 phần tử, thêm phần tử thứ 17</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Gọi add_product thêm sản phẩm thứ 17
+Kiểm tra capacity tăng từ 16 lên 32, count == 17</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Thành công: Thuật toán nhân đôi mảng động cấp phát vùng nhớ mới an toàn</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-M2-04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>REQ-6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Kiểm tra tràn số nguyên khi tính toán kích thước mở rộng (Integer Overflow in Capacity)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>current_capacity vượt ngưỡng an toàn (ví dụ: SIZE_MAX / 2)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Chạy kiểm tra SMT Z3 trên điều kiện heap_alloc_bytes
-Thực thi hàm mở rộng</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>v0: SAT (tìm được nghiệm tràn int32 cấp phát thiếu ô nhớ); v1: UNSAT</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>REQ-07, CON-04</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>H4: Cộng dồn số lượng tồn kho mới vượt trần INT_MAX</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>current_stock = 2.147.483.640, added_quantity = 20 - M3 Đô</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Gọi update_stock_quantity trên bản v0 và v1</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>v0: 2147483640 + 20 = -2147483636 (tràn số âm CWE-190); v1: từ chối trước khi cộng</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>REQ-08, CON-04</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>H4: Số lượng nhập hàng là số âm (added_quantity &lt; 0)</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity = -50 - M3 Đô</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Gọi update_stock_quantity với số lượng âm</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>v0: trừ lùi tồn kho sai nghiệp vụ; v1: phát hiện số âm từ chối an toàn</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC-09</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>REQ-09, CON-04</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>H5: Quy đổi đơn giá sản phẩm theo tỉ giá gây tràn phép nhân</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>base_price = 50.000.000, rate = 100 - M3 Đô</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Gọi scale_product_price trên bản v0 và v1</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>v0: 50.000.000 * 100 vượt INT_MAX gây tràn số (CWE-190); v1: rào chắn từ chối an toàn</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC-10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>REQ-10, CON-05</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>H6: Tranh chấp khóa phiên giữa worker nhập kho và xuất kho</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Cả 2 worker cùng giữ phiên làm việc tại h6_tranh_chap - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Chạy check_mutual_exclusion(model, 'nhap_locked', 'xuat_locked')</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>v0: vi phạm loại trừ lẫn nhau tại h6_tranh_chap (CWE-667); v1: đồng bộ mutex đạt chuẩn</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>REQ-11, REQ-12</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>H6: Double-free và Use-after-free khi giải phóng phiên kho</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>release_stock_items và close_inventory_session - M2 Trang</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Chạy kiểm toán AddressSanitizer trên bản v0 và v1</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>v0: bắt lỗi use-after-free (CWE-416) và double-free (CWE-415); v1: 0 crash ASan</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>REQ-01 đến REQ-12</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Kiểm chứng toàn luồng quản lý kho hàng kết hợp</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Mô hình kết hợp tổng thể 35 trạng thái</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Chạy chay_kiem_chung_kripke.py kiểm tra deadlock và 22 công thức CTL</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Không deadlock; v0: phát hiện lỗi tại các trạng thái vi phạm; v1: 100% thỏa mãn thuộc tính</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+Thực thi hàm calc_expand_capacity_v0 với factor lớn</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>v0: Phép nhân tràn số âm/nhỏ gây cấp phát thiếu ô nhớ; v1: Rào chắn từ chối mở rộng</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-M2-05</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mô phỏng sự cố OOM khi realloc mảng động (Fault Injection OOM NULL)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Hệ thống cạn kiệt RAM, mock_realloc trả về NULL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Ép hàm realloc trả về NULL khi mảng đầy cần mở rộng
+Quan sát phản ứng của hàm mở rộng</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>v0: Gán list = NULL làm mất sạch địa chỉ vùng nhớ cũ; v1: Trả về STATUS_ERR_ALLOC</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC-M2-06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bảo toàn địa chỉ và quyền sở hữu vùng nhớ cũ khi OOM (Ownership Retention)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>realloc trả về NULL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>So sánh địa chỉ con trỏ items trước và sau khi realloc thất bại</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>v0: Con trỏ gốc bị ghi đè thành NULL; v1: Địa chỉ cũ được bảo toàn 100%</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC-M2-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Bảo toàn tính toàn vẹn của dữ liệu đã có khi OOM (Data Integrity on Failure)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Danh sách chứa sẵn 16 mặt hàng ban đầu</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sau khi mở rộng thất bại, duyệt đọc lại 16 mặt hàng cũ</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>v0: Crash bộ nhớ do con trỏ bị NULL hóa; v1: 16 mặt hàng cũ còn nguyên vẹn</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC-M2-08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>REQ-4</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Kiểm toán rò rỉ bộ nhớ bằng LeakSanitizer (LSan Memory Leak Audit)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Biên dịch bản v0 và v1 với flag -fsanitize=leak</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Chạy kịch bản nhập kho OOM trên bản v0 và v1
+Kiểm tra log của LeakSanitizer</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>v0: LSan bắt lỗi leaked 16 blocks (CWE-401); v1: LSan báo 0 byte leaked</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TC-M2-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Con trỏ mượn bị vô hiệu hóa sau khi mảng động dời địa chỉ (Dangling Pointer on Resize)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Lưu con trỏ mượn p = find_product_by_id(&amp;list, "P0001")</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Gọi add_product kích hoạt realloc sang địa chỉ RAM mới
+Đọc dữ liệu qua con trỏ p ban đầu</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>v0: p trỏ vào vùng nhớ cũ đã bị OS thu hồi; v1: Cảnh báo Borrowed Pointer Invalidation</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TC-M2-10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Đọc con trỏ sau khi free phiên kho (Use-After-Free Audit)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Hàm cleanup_and_read_uaf_v0 giải phóng struct nhưng vẫn return *ptr</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Gọi hàm giải phóng tài nguyên phiên kho
+Thực hiện đọc/ghi vào con trỏ vừa giải phóng</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>v0: Đọc dữ liệu rác/vùng nhớ tự do (CWE-416); v1: Triệt tiêu hoàn toàn vì con trỏ đã set NULL</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TC-M2-11</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Bắt lỗi Heap-Use-After-Free bằng AddressSanitizer (ASan Crash Trigger)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Biên dịch mã nguồn với flag -fsanitize=address</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Thực thi test_sim001_heap trên bản v0
+Ghi nhận crash log do ASan sinh ra</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>v0: ASan sinh log crash: ERROR: AddressSanitizer: heap-use-after-free on address; v1: 0 crash</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TC-M2-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>REQ-5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Phòng thủ giải phóng hai lần trên cùng một con trỏ (Double-Free Defense)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Gọi product_list_free(&amp;list) liên tiếp 2 lần</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Thực hiện lệnh free(list-&gt;items) lần 1
+Thực hiện tiếp lệnh free(list-&gt;items) lần 2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>v0: Crash OS double free or corruption (CWE-415); v1: Lần 2 gặp con trỏ NULL nên bỏ qua an toàn</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TC-M2-13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>REQ-3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Kiểm toán bất biến an toàn bộ nhớ (Safety Invariant: count &lt;= capacity)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Chạy qua 50 lần thêm/xóa ngẫu nhiên</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Kiểm tra điều kiện list.count &lt;= list.capacity tại mọi thời điểm</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bất biến an toàn luôn được duy trì 100% trong suốt vòng đời mảng động</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TC-M2-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-2, REQ-3, REQ-4, REQ-5</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Kiểm thử hồi quy đối chứng toàn diện pytest (Regression Verification Suite)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Bộ test pytest test_verify_v0_cases_on_v1.py</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Chạy toàn bộ test cases trên bản lỗi v0
+Chạy lại toàn bộ test cases trên bản vá v1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>v0: Phát hiện đầy đủ lỗi CWE-190, CWE-401, CWE-416; v1: 100% PASSED (Xanh toàn bộ)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TC-M3-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>REQ-1, REQ-4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cộng dồn số lượng hàng hóa gây tràn số nguyên có dấu 32-bit</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>old_stock = 2.147.483.640, added_quantity = 100</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Chạy check_satisfiability() trên stock_addition_overflow (Chương 3 Z3)
+Kiểm tra AG(!integer_overflow) trên luồng M3-v0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>v0: VI PHẠM (CWE-190 Signed Integer Overflow), kết quả lật âm; v1: ĐÚNG (chặn trước khi cộng)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TC-M3-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>REQ-3, REQ-5</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Từ chối số lượng nhập hàng là số âm</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>added_quantity = -50</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Kiểm tra AG(!negative_input) trên luồng M3-v0
+Kiểm tra lại trên luồng M3-v1</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>v0: VI PHẠM (nhận số âm); v1: ĐÚNG (rào chắn từ chối ngay lập tức)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2956,253 +3566,225 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ingest_raw_line</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>buffer_copy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>dst, cap, raw_line</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>raw_line</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>32</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>buffer-overflow</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>H1 — Nạp chuỗi vào bộ đệm stack 32 byte (M1 Thọ)</t>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>H1 — Nạp chuỗi vào bộ đệm stack 32 byte bằng strcpy (M1 Thọ - CWE-120/121)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>get_token_field</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>array_read</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>token_offsets, token_count, field_idx</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>out-of-bounds-read</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>H2 — Đọc trường token theo chỉ số mảng (M1 Thọ)</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>arithmetic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>token_count, field_idx</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>integer-overflow</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>H2 — Phép toán chỉ số trường token mảng (M1 Thọ - CWE-125/190)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>expand_stock_items</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>list, new_capacity</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>16</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>memory-leak</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>H3 — realloc mở rộng mảng khi OOM gây rò rỉ bộ nhớ (M2 Trang)</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>H3 — realloc mở rộng mảng khi OOM gây rò rỉ bộ nhớ (M2 Trang - CWE-401)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>release_stock_items</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>alloc_release</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>list</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>16</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>use-after-free</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>H6 — free() không gán NULL dẫn tới Use-After-Free (M2 Trang)</t>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>H6 — free() không gán NULL dẫn tới Use-After-Free (M2 Trang - CWE-416)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>update_stock_quantity</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>arithmetic</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>current_stock, added_quantity</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>integer-overflow</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>H4 — Cộng dồn tồn kho tràn signed int 32-bit (M3 Đô)</t>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>H4 — Cộng dồn tồn kho tràn signed int 32-bit (M3 Đô - CWE-190)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>scale_product_price</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>arithmetic</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>base_price, rate</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>integer-overflow</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>H5 — Nhân tỉ giá quy đổi tràn int32 (M3 Đô)</t>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>H5 — Nhân tỉ giá quy đổi tràn int32 (M3 Đô - CWE-190)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>calc_batch_capacity</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>python</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>divide</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>total_items, batch_size</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>divide-by-zero</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>H3 — Chia cho 0 khi batch_size = 0 (black-box fuzz)</t>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>H3 — Chia cho 0 khi batch_size = 0 (M2 Trang - Black-box Fuzzing)</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3255,110 +3837,164 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>buffer_capacity_check</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cap, input_len</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>cap == 32 and input_len &gt;= cap</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>input_len - cap</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>H1 — Kiểm tra dung lượng bộ đệm stack 32 byte (M1 Thọ - CWE-120)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>token_index_check</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>token_count, field_idx</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>token_count &gt; 0 and (field_idx &lt; 0 or field_idx &gt;= token_count)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>field_idx - token_count</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>H2 — Kiểm tra chỉ số mảng token [0, token_count - 1] (M1 Thọ - CWE-125)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>heap_alloc_bytes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>new_capacity, item_size</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>new_capacity &gt;= 1 and item_size == 48 and new_capacity * item_size &gt; 2147483647</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>new_capacity * item_size</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>H3 — Kích thước tái cấp phát Heap vượt 2GB khi new_capacity lớn (M2 Trang - CWE-190)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>stock_addition_overflow</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>current_stock, added_quantity</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>current_stock &gt;= 0 and current_stock &lt;= 2147483647 and added_quantity &gt;= 1 and added_quantity &lt;= 2147483647 and current_stock + added_quantity &gt; 2147483647</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>current_stock + added_quantity</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>H4 — phép cộng dồn tồn kho mới vào tồn kho cũ vượt trần INT_MAX (M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>heap_alloc_bytes</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity, item_size</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity &gt;= 1 and item_size == 48 and new_capacity * item_size &gt; 2147483647</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>new_capacity * item_size</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>H3 — kích thước tái cấp phát Heap vượt 2GB khi new_capacity lớn (M2 Trang)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>old_stock, added_quantity</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>old_stock &gt;= 0 and old_stock &lt;= 2147483647 and added_quantity &gt;= 1 and added_quantity &lt;= 2147483647 and old_stock + added_quantity &gt; 2147483647</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>old_stock + added_quantity</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>H4 — Phép cộng dồn tồn kho mới vào tồn kho cũ vượt trần INT_MAX (M3 Đô - CWE-190)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>negative_quantity_check</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>added_quantity</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>added_quantity &lt; 0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>added_quantity</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>H4 — Số lượng nhập hàng là số âm làm sai lệch số liệu kho (M3 Đô)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>price_multiplication_overflow</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>base_price, rate</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>base_price &gt; 0 and rate &gt; 1 and base_price * rate &gt; 2147483647</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>base_price * rate</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>H5 — phép nhân đơn giá x tỉ giá quy đổi tràn int32 (M3 Đô)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>negative_quantity_check</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity &lt; 0</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>added_quantity</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>H4 — số lượng nhập hàng là số âm làm sai lệch số liệu kho (M3 Đô)</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>H5 — Phép nhân đơn giá x tỉ giá quy đổi tràn int32 (M3 Đô - CWE-190)</t>
         </is>
       </c>
     </row>

</xml_diff>